<commit_message>
Polish mage spell visuals and preserve cast state during equipment changes
Replace per-cast JSON cloning and synchronous counter writes with isolated snapshots and coalesced background persistence. Preserve skill and slot cooldowns through equip swaps. Add sky starfall, airborne void pull, opaque animated meteor, large storm lightning and clearer persistent fields while retaining stable skill IDs.

Validated all ten effects on Android, 186 mage checks, 13 combat/persistence checks and a 90-second five-spell automatic casting sample.
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R5697e4c162fa410a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rcdd652f826014c95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R1ea966fae57e4c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="Ra35561e77f654be2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="Rc9b8aaca119640cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rf1541473b98a4baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="7" r:id="R8ad4982abf744c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rb0ff7fc8f78f4512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R24806a1170ea4227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="Rd2db2859eb1143e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R0b53755e09a54b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R08c34fcb527b40d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R127dde07212e4472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R8e0c3b3c278c492e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rce18cac80b4c4040"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -311,7 +312,19 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Mage_Guide" displayName="Mage_Guide" ref="A1:B20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Mage_Targeting" displayName="Mage_Targeting" ref="A1:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="SkillId"/>
+    <x:tableColumn id="2" name="지점 선택"/>
+    <x:tableColumn id="3" name="판정과 대상"/>
+    <x:tableColumn id="4" name="표시 순서"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Mage_Guide" displayName="Mage_Guide" ref="A1:B22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Description"/>
@@ -653,10 +666,10 @@
         <x:v>ArcaneVolley</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>비전 탄막</x:v>
+        <x:v>유성우</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>추적 투사체</x:v>
+        <x:v>전장 낙하</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:v>62</x:v>
@@ -671,7 +684,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
-        <x:v>추적 탄환을 연속 발사합니다. 적을 쓰러뜨리면 다음 적을 노립니다.</x:v>
+        <x:v>전장 곳곳의 적에게 별빛을 차례로 떨어뜨립니다. 별빛이 닿은 적에게 피해를 줍니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="70" customHeight="1">
@@ -845,13 +858,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="I11" s="5" t="str">
-        <x:v>적을 끌어모아 이동 속도를 20% 낮추고 지속 피해를 줍니다. 마지막에 균열이 폭발합니다. 보스는 끌어당기지 못합니다.</x:v>
+        <x:v>적이 모인 곳의 허공에 원형 균열을 엽니다. 균열 안의 적을 중심으로 끌어당기며 지속 피해를 주고, 닫힐 때 폭발합니다. 보스는 끌어당기지 못합니다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b338307a1bc41bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bbf21c663404b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1028,7 +1041,7 @@
         <x:v>FireTornado</x:v>
       </x:c>
       <x:c r="C4" s="18" t="n">
-        <x:v>0.800000011920929</x:v>
+        <x:v>0.8500000238418579</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
         <x:v>5</x:v>
@@ -1076,7 +1089,7 @@
         <x:v>ArcaneVolley</x:v>
       </x:c>
       <x:c r="C5" s="18" t="n">
-        <x:v>0.10000000149011612</x:v>
+        <x:v>0.550000011920929</x:v>
       </x:c>
       <x:c r="D5" s="18" t="n">
         <x:v>1.3199999332427979</x:v>
@@ -1122,7 +1135,7 @@
         <x:v>VenomMist</x:v>
       </x:c>
       <x:c r="C6" s="18" t="n">
-        <x:v>1.25</x:v>
+        <x:v>1.399999976158142</x:v>
       </x:c>
       <x:c r="D6" s="18" t="n">
         <x:v>4.5</x:v>
@@ -1260,7 +1273,7 @@
         <x:v>Sanctuary</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
-        <x:v>1.7000000476837158</x:v>
+        <x:v>1.899999976158142</x:v>
       </x:c>
       <x:c r="D9" s="18" t="n">
         <x:v>4.199999809265137</x:v>
@@ -1306,7 +1319,7 @@
         <x:v>Meteor</x:v>
       </x:c>
       <x:c r="C10" s="18" t="n">
-        <x:v>1.350000023841858</x:v>
+        <x:v>1.5499999523162842</x:v>
       </x:c>
       <x:c r="D10" s="18" t="n">
         <x:v>0.800000011920929</x:v>
@@ -1352,7 +1365,7 @@
         <x:v>VoidRift</x:v>
       </x:c>
       <x:c r="C11" s="18" t="n">
-        <x:v>1.600000023841858</x:v>
+        <x:v>1.2999999523162842</x:v>
       </x:c>
       <x:c r="D11" s="18" t="n">
         <x:v>3</x:v>
@@ -1392,7 +1405,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f957c6c4a94948"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8318e813f2de42f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1582,7 +1595,7 @@
       </x:c>
       <x:c r="B5" s="16" t="str">
         <x:f>'Skills'!C5</x:f>
-        <x:v>비전 탄막</x:v>
+        <x:v>유성우</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>미정</x:v>
@@ -1810,7 +1823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24e44b919d1e4856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc042dbc38d4e4c13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1983,7 +1996,7 @@
       </x:c>
       <x:c r="B5" s="16" t="str">
         <x:f>'Skills'!C5</x:f>
-        <x:v>비전 탄막</x:v>
+        <x:v>유성우</x:v>
       </x:c>
       <x:c r="C5" s="9" t="n">
         <x:v>30</x:v>
@@ -2239,7 +2252,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f86bd596c1b4de2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f054e3116543f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4495,7 +4508,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd578b68dc8874a0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa243002569d4cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4824,12 +4837,187 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d8085174344f21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa305743c1c49b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2D6176"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>SkillId</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>지점 선택</x:v>
+      </x:c>
+      <x:c r="C1" s="8" t="str">
+        <x:v>판정과 대상</x:v>
+      </x:c>
+      <x:c r="D1" s="8" t="str">
+        <x:v>표시 순서</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="68" customHeight="1">
+      <x:c r="A2" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B2" s="5" t="str">
+        <x:v>적이 가장 많이 모인 지점</x:v>
+      </x:c>
+      <x:c r="C2" s="5" t="str">
+        <x:v>지정 지점 고정 원형 범위 · 천벌은 가장자리/HUD 안쪽 보정</x:v>
+      </x:c>
+      <x:c r="D2" s="5" t="str">
+        <x:v>즉발 낙뢰 전면 · 구름 전면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="68" customHeight="1">
+      <x:c r="A3" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="str">
+        <x:v>전장의 유효 적 순회</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="str">
+        <x:v>개화는 시전 시작 시 단일/다수 분기</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="str">
+        <x:v>빙정 전면 · 바닥 예고 후면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="68" customHeight="1">
+      <x:c r="A4" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>현재 중심에 가까운 살아 있는 적 추적</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>이동 장판 안 최대 3체</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>지속 장판 후면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="68" customHeight="1">
+      <x:c r="A5" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="str">
+        <x:v>전장 내 적을 차례로 선택</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="str">
+        <x:v>별빛은 선택 순간 위치로 낙하 · 회피 가능</x:v>
+      </x:c>
+      <x:c r="D5" s="5" t="str">
+        <x:v>낙하와 충돌 전면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="68" customHeight="1">
+      <x:c r="A6" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="str">
+        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="str">
+        <x:v>고정 장판 안 최대 5체 · 틱마다 재판정</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="str">
+        <x:v>지속 장판 후면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="68" customHeight="1">
+      <x:c r="A7" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="str">
+        <x:v>적이 가장 많이 모인 지점</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="str">
+        <x:v>고정 범위 최대 4체</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>바닥 예고 후면 · 솟는 바위 전면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="68" customHeight="1">
+      <x:c r="A8" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>유효 표적 방향으로 관통 경로 설정</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="str">
+        <x:v>경로 안 최대 5체</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>단발 파동 전면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="68" customHeight="1">
+      <x:c r="A9" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="str">
+        <x:v>생존 아군 중 HP 비율 최저</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="str">
+        <x:v>매 회복마다 대상 재선정</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="str">
+        <x:v>성역 후면 · 회복 반짝임 전면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="68" customHeight="1">
+      <x:c r="A10" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="str">
+        <x:v>예고 위치 고정 · 충돌 후 잔불 2회</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="str">
+        <x:v>운석과 폭발 전면 · 잔불 후면</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="68" customHeight="1">
+      <x:c r="A11" s="9" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="str">
+        <x:v>허공 원 안 몸체 중심만 흡인 · 보스 흡인 면역</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="str">
+        <x:v>지속 균열 후면 · 붕괴 전면</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8c52c43f33d4793"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF70858C"/>
@@ -4850,160 +5038,176 @@
     </x:row>
     <x:row r="2" ht="62" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>용도</x:v>
+        <x:v>편성 조작</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>개발자 열람용 스킬 카탈로그입니다. 현재 런타임 원본은 MageTowerSkillList와 각 MageTowerSkillSO입니다. 이 파일의 편집 내용은 자동으로 게임에 반영되지 않습니다.</x:v>
+        <x:v>슬롯 선택 → 스킬 선택 → 장착 또는 교체. 다른 슬롯의 스킬을 고르면 원자적으로 자리 바꾸기. 해제·교체는 진행 중인 효과를 취소하지 않으며 슬롯 및 스킬 쿨타임을 모두 보존합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>수정 절차</x:v>
+        <x:v>시전 기록</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>스킬 데이터와 동작을 수정한 뒤 카탈로그를 함께 갱신합니다. 향후 임포터 연결 시 SkillId와 Key를 고정 키로 사용하고 수치 검증 후 데이터베이스를 교체합니다.</x:v>
+        <x:v>스킬 시전 카운터는 메모리에 즉시 반영하고 짧게 묶어 비동기로 저장합니다. 재화 거래는 앞선 저장 완료를 확인한 뒤 기록하며 앱 백그라운드와 계정 전환에서 남은 카운터를 저장합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>버전</x:v>
+        <x:v>용도</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>게임 0.9.0 · 스킬 데이터 계약 mage-2 · 스킬 ID 0~9. 기존 0~2와 에셋 GUID를 유지했습니다.</x:v>
+        <x:v>개발자 열람용 스킬 카탈로그입니다. 현재 런타임 원본은 MageTowerSkillList와 각 MageTowerSkillSO입니다. 이 파일의 편집 내용은 자동으로 게임에 반영되지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" s="5" t="str">
-        <x:v>단위</x:v>
+        <x:v>수정 절차</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>BasePower는 강화 전 한 번의 피해 또는 회복량입니다. RadiusWU는 월드 단위입니다. Bloom 배율은 강화·각성을 반영한 1회 효과량에 곱합니다.</x:v>
+        <x:v>스킬 데이터와 동작을 수정한 뒤 카탈로그를 함께 갱신합니다. 향후 임포터 연결 시 SkillId와 Key를 고정 키로 사용하고 수치 검증 후 데이터베이스를 교체합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" s="5" t="str">
-        <x:v>공통 성장</x:v>
+        <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>직접 강화 E는 비전 지식으로 0~100, 각성 A는 동일 스킬 파편으로 0~10. A4/A8에 각각 1회 추가(화염 회오리는 2틱), A마다 효과량 +5%와 쿨타임 -2%. 운석은 고정 1회 충돌과 잔불 2회이며 타격 수 보너스를 사용하지 않습니다.</x:v>
+        <x:v>게임 0.10.0 · 스킬 데이터 계약 mage-3 · 스킬 ID 0~9. 기존 0~2와 에셋 GUID를 유지했습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" s="5" t="str">
-        <x:v>개화 저장</x:v>
+        <x:v>단위</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>A10에서 해금되며 기본은 꺼짐입니다. 마탑 상세에서 전환하고 다음 시전부터 적용합니다. 진행 중인 시전의 배율·대상 조건·쿨타임은 바뀌지 않습니다.</x:v>
+        <x:v>BasePower는 강화 전 한 번의 피해 또는 회복량입니다. RadiusWU는 월드 단위입니다. Bloom 배율은 강화·각성을 반영한 1회 효과량에 곱합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" s="5" t="str">
-        <x:v>회복과 전투력</x:v>
+        <x:v>공통 성장</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>회복의 성역은 살아있는 아군 중 HP 비율이 가장 낮은 대상을 반복 회복합니다. 전원이 HP 90% 이상이면 자동 시전을 보류합니다. 회복·제어 효용은 단일 대상 DPS 기반 전투력에 더하지 않습니다.</x:v>
+        <x:v>직접 강화 E는 비전 지식으로 0~100, 각성 A는 동일 스킬 파편으로 0~10. A4/A8에 각각 1회 추가(화염 회오리는 2틱), A마다 효과량 +5%와 쿨타임 -2%. 운석은 고정 1회 충돌과 잔불 2회이며 타격 수 보너스를 사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>확률</x:v>
+        <x:v>개화 저장</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>전체 뽑기는 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 스킬 10종은 등급 없이 각각 5%로 획득합니다. 희귀도는 장비에만 적용합니다.</x:v>
+        <x:v>A10에서 해금되며 기본은 꺼짐입니다. 마탑 상세에서 전환하고 다음 시전부터 적용합니다. 진행 중인 시전의 배율·대상 조건·쿨타임은 바뀌지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>파편</x:v>
+        <x:v>회복과 전투력</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>첫 획득은 해금만 지급합니다. 모든 스킬의 중복 뽑기는 30파편입니다. 메인 최초 보상의 기존 중복 대체 및 명시적 파편 보상은 1개 단위를 유지합니다.</x:v>
+        <x:v>회복의 성역은 살아있는 아군 중 HP 비율이 가장 낮은 대상을 반복 회복합니다. 전원이 HP 90% 이상이면 자동 시전을 보류합니다. 회복·제어 효용은 단일 대상 DPS 기반 전투력에 더하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>투자 기간</x:v>
+        <x:v>확률</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>각성 누적55파편 기준입니다. 주당21회 전부 마탑에 사용하고 최초 보상·기존 파편을 제외하면 미보유 특정 스킬의 평균 개화 기간은 60회 뽑기, 약2.86주입니다. 장비 뽑기에 주화를 나누면 더 오래 걸립니다.</x:v>
+        <x:v>전체 뽑기는 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 스킬 10종은 등급 없이 각각 5%로 획득합니다. 희귀도는 장비에만 적용합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>확률 편차</x:v>
+        <x:v>파편</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>Acquisition의 P90은 해당 횟수까지 약90%가 목표를 달성한다는 정확한 음이항 계산입니다. 스킬당105회(약5주). 천장과 기간 보장은 없으며 수 주는 평균 목표입니다.</x:v>
+        <x:v>첫 획득은 해금만 지급합니다. 모든 스킬의 중복 뽑기는 30파편입니다. 메인 최초 보상의 기존 중복 대체 및 명시적 파편 보상은 1개 단위를 유지합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>특수 개화</x:v>
+        <x:v>투자 기간</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>천벌은 약2초 예고 후 큰 범위의 최대10체를 공격합니다. 실제 반경은 뷰포트 폭의1/4을 월드 단위1.6~2.6으로 제한합니다. 만년빙정은 시전 시작 시 화면 내 유효 적 1체 여부로 단일/다수 형태를 선택합니다.</x:v>
+        <x:v>각성 누적55파편 기준입니다. 주당21회 전부 마탑에 사용하고 최초 보상·기존 파편을 제외하면 미보유 특정 스킬의 평균 개화 기간은 60회 뽑기, 약2.86주입니다. 장비 뽑기에 주화를 나누면 더 오래 걸립니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>최적화</x:v>
+        <x:v>확률 편차</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>아이콘48px·16색 이내·Point. Atlas_UIPixel ASTC4×4. VFX는 공유 시트와 사전 생성 AnimationClip·프리팹을 사용하고 Atlas_MageVFX에 포함합니다. 저사양은 동시 얼음 연출만 줄이고 피해 수는 유지합니다.</x:v>
+        <x:v>Acquisition의 P90은 해당 횟수까지 약90%가 목표를 달성한다는 정확한 음이항 계산입니다. 스킬당105회(약5주). 천장과 기간 보장은 없으며 수 주는 평균 목표입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>개화 아이콘</x:v>
+        <x:v>특수 개화</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>개화 ON이면 BloomIcon을 사용합니다. 기본 실루엣과 구도를 유지하고 작은 발광·색조만 변화합니다. OFF 및 미해금 상태는 원본 아이콘을 사용합니다.</x:v>
+        <x:v>천벌은 약2초 예고 후 큰 범위의 최대10체를 공격합니다. 실제 반경은 뷰포트 폭의1/4을 월드 단위1.6~2.6으로 제한합니다. 만년빙정은 시전 시작 시 화면 내 유효 적 1체 여부로 단일/다수 형태를 선택합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>타격 연출</x:v>
+        <x:v>최적화</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>피해·피격 반응·효과음은 스프라이트의 적중 프레임에 맞춥니다. 일회 연출은 반복하지 않으며, 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
+        <x:v>아이콘48px·16색 이내·Point. Atlas_UIPixel ASTC4×4. VFX는 공유 시트와 사전 생성 AnimationClip·프리팹을 사용하고 Atlas_MageVFX에 포함합니다. 저사양은 동시 얼음 연출만 줄이고 피해 수는 유지합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="62" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>외부 원본</x:v>
+        <x:v>개화 아이콘</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>ExternalAssets는 원본 저장소이며 직접 변경하지 않습니다. Assets 탭의 작업본만 게임에서 사용합니다. 출처 및 생성 공정은 AI/comfyui/mage-skills/20260915 및20260916 기록을 따릅니다.</x:v>
+        <x:v>개화 ON이면 BloomIcon을 사용합니다. 기본 실루엣과 구도를 유지하고 작은 발광·색조만 변화합니다. OFF 및 미해금 상태는 원본 아이콘을 사용합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="62" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>서버 계약</x:v>
+        <x:v>타격 연출</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>MageSkillStateSnapshot schema1은 catalogVersion·progressionRevision·정렬된 스킬 상태·장착 ID를 내보냅니다. 기존 계정/권한/전체 저장 리비전 계약과 함께 사용해야 합니다. 서버 응답을 적용하는 기능은 추가하지 않았습니다.</x:v>
+        <x:v>피해·피격 반응·효과음은 스프라이트의 적중 프레임에 맞춥니다. 일회 연출은 반복하지 않으며, 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="62" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>레거시 코드</x:v>
+        <x:v>외부 원본</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>64비트 packed code는 개화를 담지 못하고 파편 상한65535입니다. 범위를 넘으면 예외로 거부하며 새 스냅샷을 사용합니다. 기존 저장 JSON의 BloomEnabled 누락은 false로 읽습니다.</x:v>
+        <x:v>ExternalAssets는 원본 저장소이며 직접 변경하지 않습니다. Assets 탭의 작업본만 게임에서 사용합니다. 출처 및 생성 공정은 AI/comfyui/mage-skills/20260915 및20260916-combat 기록을 따릅니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
       <x:c r="A20" s="5" t="str">
+        <x:v>서버 계약</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="str">
+        <x:v>MageSkillStateSnapshot schema1은 catalogVersion·progressionRevision·정렬된 스킬 상태·장착 ID를 내보냅니다. 기존 계정/권한/전체 저장 리비전 계약과 함께 사용해야 합니다. 서버 응답을 적용하는 기능은 추가하지 않았습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="62" customHeight="1">
+      <x:c r="A21" s="5" t="str">
+        <x:v>레거시 코드</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="str">
+        <x:v>64비트 packed code는 개화를 담지 못하고 파편 상한65535입니다. 범위를 넘으면 예외로 거부하며 새 스냅샷을 사용합니다. 기존 저장 JSON의 BloomEnabled 누락은 false로 읽습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="62" customHeight="1">
+      <x:c r="A22" s="5" t="str">
         <x:v>보류 개화</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="str">
+      <x:c r="B22" s="5" t="str">
         <x:v>천벌·만년빙정 외 8종은 개화 미정으로 표기합니다. 현재는 기존 피해 또는 회복의15% 증가만 적용하며 확정된 고유 개화로 오해하지 않도록 유지합니다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R350e59f2384a4db4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0e0f27093e4d00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Polish combat impacts, crowd control, and mage tower effects
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rb0ff7fc8f78f4512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R24806a1170ea4227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="Rd2db2859eb1143e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R0b53755e09a54b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R08c34fcb527b40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R127dde07212e4472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R8e0c3b3c278c492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rce18cac80b4c4040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R5fec058bdb964bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R9965d484d4754f36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R14d5c4838099422b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R6e313ad36a9e4994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R132f15671c6848ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R0f0ccff8863e4ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Reff0faa5f516437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R70b674a9002e4db8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -864,7 +864,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bbf21c663404b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912139e06cfc4334"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1405,7 +1405,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8318e813f2de42f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fc8405df4b44b04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1510,10 +1510,10 @@
       <x:c r="K2" s="5"/>
       <x:c r="L2" s="5"/>
       <x:c r="M2" s="9" t="n">
-        <x:v>1.6</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="N2" s="9" t="n">
-        <x:v>2.6</x:v>
+        <x:v>2.1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="90" customHeight="1">
@@ -1823,7 +1823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc042dbc38d4e4c13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9efe7a4b140c4cc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2252,7 +2252,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f054e3116543f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77fad7a1690a4689"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4508,7 +4508,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa243002569d4cdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c402cd58564257"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4837,7 +4837,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa305743c1c49b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488c3cb391bc44fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,7 +4869,7 @@
         <x:v>표시 순서</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="68" customHeight="1">
+    <x:row r="2" ht="76" customHeight="1">
       <x:c r="A2" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -4877,13 +4877,14 @@
         <x:v>적이 가장 많이 모인 지점</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>지정 지점 고정 원형 범위 · 천벌은 가장자리/HUD 안쪽 보정</x:v>
+        <x:v>고정 원형 범위 · 천벌의 구름 높이와 벼락 길이는 상단 여백에 맞춤
+연출 높이 보정으로 타격 지점을 아래로 이동하지 않음</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
         <x:v>즉발 낙뢰 전면 · 구름 전면</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="68" customHeight="1">
+    <x:row r="3" ht="76" customHeight="1">
       <x:c r="A3" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -4897,7 +4898,7 @@
         <x:v>빙정 전면 · 바닥 예고 후면</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="68" customHeight="1">
+    <x:row r="4" ht="76" customHeight="1">
       <x:c r="A4" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -4911,7 +4912,7 @@
         <x:v>지속 장판 후면</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="68" customHeight="1">
+    <x:row r="5" ht="76" customHeight="1">
       <x:c r="A5" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -4919,13 +4920,14 @@
         <x:v>전장 내 적을 차례로 선택</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>별빛은 선택 순간 위치로 낙하 · 회피 가능</x:v>
+        <x:v>별빛은 비행 전반 70% 동안 대상을 추적한 뒤 낙하 지점을 확정
+0.22초 간격 · 비행 0.48초</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
         <x:v>낙하와 충돌 전면</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="68" customHeight="1">
+    <x:row r="6" ht="76" customHeight="1">
       <x:c r="A6" s="9" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -4933,13 +4935,13 @@
         <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>고정 장판 안 최대 5체 · 틱마다 재판정</x:v>
+        <x:v>고정 장판 안 최대 5체 · 틱마다 재판정 · 감속 25%, 기절과 별도 유지</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
         <x:v>지속 장판 후면</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="68" customHeight="1">
+    <x:row r="7" ht="76" customHeight="1">
       <x:c r="A7" s="9" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -4947,13 +4949,13 @@
         <x:v>적이 가장 많이 모인 지점</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
-        <x:v>고정 범위 최대 4체</x:v>
+        <x:v>고정 범위 최대 4체 · 기절이 기존 감속을 지우지 않음</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
         <x:v>바닥 예고 후면 · 솟는 바위 전면</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="68" customHeight="1">
+    <x:row r="8" ht="76" customHeight="1">
       <x:c r="A8" s="9" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -4961,13 +4963,13 @@
         <x:v>유효 표적 방향으로 관통 경로 설정</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>경로 안 최대 5체</x:v>
+        <x:v>파동이 실제 통과한 경로 안 최대 5체 · 파동당 같은 적 1회</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
         <x:v>단발 파동 전면</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="68" customHeight="1">
+    <x:row r="9" ht="76" customHeight="1">
       <x:c r="A9" s="9" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -4981,7 +4983,7 @@
         <x:v>성역 후면 · 회복 반짝임 전면</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="68" customHeight="1">
+    <x:row r="10" ht="76" customHeight="1">
       <x:c r="A10" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -4995,7 +4997,7 @@
         <x:v>운석과 폭발 전면 · 잔불 후면</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="68" customHeight="1">
+    <x:row r="11" ht="76" customHeight="1">
       <x:c r="A11" s="9" t="n">
         <x:v>9</x:v>
       </x:c>
@@ -5003,7 +5005,8 @@
         <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
-        <x:v>허공 원 안 몸체 중심만 흡인 · 보스 흡인 면역</x:v>
+        <x:v>허공 원 안 몸체 중심만 흡인 · 보스 흡인 면역
+약한 감속으로 기존 강한 감속을 덮어쓰지 않음</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
         <x:v>지속 균열 후면 · 붕괴 전면</x:v>
@@ -5012,7 +5015,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8c52c43f33d4793"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e6369b610a4dcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5073,7 +5076,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.10.0 · 스킬 데이터 계약 mage-3 · 스킬 ID 0~9. 기존 0~2와 에셋 GUID를 유지했습니다.</x:v>
+        <x:v>게임 0.10.2 · 스킬 데이터 계약 mage-3 · 스킬 ID 0~9와 기존 에셋 GUID를 유지합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -5140,12 +5143,12 @@
         <x:v>Acquisition의 P90은 해당 횟수까지 약90%가 목표를 달성한다는 정확한 음이항 계산입니다. 스킬당105회(약5주). 천장과 기간 보장은 없으며 수 주는 평균 목표입니다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="62" customHeight="1">
+    <x:row r="15" ht="84" customHeight="1">
       <x:c r="A15" s="5" t="str">
         <x:v>특수 개화</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>천벌은 약2초 예고 후 큰 범위의 최대10체를 공격합니다. 실제 반경은 뷰포트 폭의1/4을 월드 단위1.6~2.6으로 제한합니다. 만년빙정은 시전 시작 시 화면 내 유효 적 1체 여부로 단일/다수 형태를 선택합니다.</x:v>
+        <x:v>천벌은 약 2초 예고 후 고정 반경 2.1 월드 단위 안 최대 10체를 공격합니다. 기기 비율이 피해 범위를 바꾸지 않습니다. Bloom의 최소·최대 반경은 모두 2.1입니다. 만년빙정은 시전 시작 시 유효 적 1체 여부로 단일/다수 형태를 선택합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
@@ -5164,20 +5167,20 @@
         <x:v>개화 ON이면 BloomIcon을 사용합니다. 기본 실루엣과 구도를 유지하고 작은 발광·색조만 변화합니다. OFF 및 미해금 상태는 원본 아이콘을 사용합니다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="62" customHeight="1">
+    <x:row r="18" ht="84" customHeight="1">
       <x:c r="A18" s="5" t="str">
         <x:v>타격 연출</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>피해·피격 반응·효과음은 스프라이트의 적중 프레임에 맞춥니다. 일회 연출은 반복하지 않으며, 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="62" customHeight="1">
+        <x:v>타격 시점에 피해·피격 반응·효과음을 맞춥니다. 별빛은 겹쳐 낙하하고 운석은 충돌 후 잔불을 남깁니다. 기절과 감속은 독립 만료하며 감속은 합산하지 않고 가장 강한 효과만 적용합니다. 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="84" customHeight="1">
       <x:c r="A19" s="5" t="str">
         <x:v>외부 원본</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>ExternalAssets는 원본 저장소이며 직접 변경하지 않습니다. Assets 탭의 작업본만 게임에서 사용합니다. 출처 및 생성 공정은 AI/comfyui/mage-skills/20260915 및20260916-combat 기록을 따릅니다.</x:v>
+        <x:v>ExternalAssets는 원본 저장소이며 직접 변경하지 않습니다. Assets 탭의 작업본만 사용합니다. 생성 출처는 AI/comfyui/mage-skills/20260915, 20260916-combat 및 20260917-polish입니다. 운석 잔흔은 두 모델 비교 후 채택한 단일 64px·6색 지면 데칼입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -5207,7 +5210,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b0e0f27093e4d00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6882e447a3e4987"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix progression blockers and improve mobile playability
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R5fec058bdb964bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R9965d484d4754f36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R14d5c4838099422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R6e313ad36a9e4994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R132f15671c6848ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R0f0ccff8863e4ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Reff0faa5f516437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R70b674a9002e4db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Re32e84b2bce343ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R7e85d5c0db3a4613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R8a02e866d6fb41da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R4ea15bbc3c7c46b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R91ce146a850c4c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R4c4b104688a949c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R2bfd5c4faade442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R6f00d504520941a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -695,7 +695,7 @@
         <x:v>VenomMist</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>맹독 안개</x:v>
+        <x:v>맹독 늪</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
         <x:v>지속 둔화</x:v>
@@ -713,7 +713,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I6" s="5" t="str">
-        <x:v>독 안개로 지속 피해를 주고 이동 속도를 25% 낮춥니다.</x:v>
+        <x:v>맹독 늪을 펼쳐 범위 안의 적에게 지속 피해를 주고 이동 속도를 25% 낮춥니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="70" customHeight="1">
@@ -800,7 +800,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="I9" s="5" t="str">
-        <x:v>체력 비율이 가장 낮은 왕국군을 반복해서 회복합니다.</x:v>
+        <x:v>성역을 펼쳐 범위 안에서 체력 비율이 가장 낮은 왕국군을 반복해서 회복합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="70" customHeight="1">
@@ -864,7 +864,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R912139e06cfc4334"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7912bafa8f142b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1405,7 +1405,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fc8405df4b44b04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccbff2996eec4f5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1628,7 +1628,7 @@
       </x:c>
       <x:c r="B6" s="16" t="str">
         <x:f>'Skills'!C6</x:f>
-        <x:v>맹독 안개</x:v>
+        <x:v>맹독 늪</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
         <x:v>미정</x:v>
@@ -1823,7 +1823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9efe7a4b140c4cc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2101a43777c74708"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2033,7 +2033,7 @@
       </x:c>
       <x:c r="B6" s="16" t="str">
         <x:f>'Skills'!C6</x:f>
-        <x:v>맹독 안개</x:v>
+        <x:v>맹독 늪</x:v>
       </x:c>
       <x:c r="C6" s="9" t="n">
         <x:v>30</x:v>
@@ -2252,7 +2252,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77fad7a1690a4689"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R422a35627e2648dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4508,7 +4508,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c402cd58564257"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e724c77b5947fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4837,7 +4837,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R488c3cb391bc44fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0294a0713b664c4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5015,7 +5015,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e6369b610a4dcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f77bf989dcb433c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5210,7 +5210,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6882e447a3e4987"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774af23012b741fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve mage manual casting, awakening details and spell visuals
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Re32e84b2bce343ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R7e85d5c0db3a4613"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R8a02e866d6fb41da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R4ea15bbc3c7c46b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R91ce146a850c4c4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R4c4b104688a949c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R2bfd5c4faade442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R6f00d504520941a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rd3e087a157ec40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R81dbcc681f6a44d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R6149853889ba41a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R9ab34a80bdb54e67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="Re554c98a7e904d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R324efd102463456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rd777cf03eb074eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R076e2cb4d77c4608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Mage_Skills" displayName="Mage_Skills" ref="A1:I11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Mage_Skills" displayName="Mage_Skills" ref="A1:I10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="Key"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Mage_Parameters" displayName="Mage_Parameters" ref="A1:O11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Mage_Parameters" displayName="Mage_Parameters" ref="A1:O10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="Key"/>
@@ -238,7 +238,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Mage_Bloom" displayName="Mage_Bloom" ref="A1:N11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Mage_Bloom" displayName="Mage_Bloom" ref="A1:N10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="스킬"/>
@@ -260,7 +260,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Mage_Acquisition" displayName="Mage_Acquisition" ref="A1:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Mage_Acquisition" displayName="Mage_Acquisition" ref="A1:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="스킬"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Mage_Assets" displayName="Mage_Assets" ref="A1:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Mage_Assets" displayName="Mage_Assets" ref="A1:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="Key"/>
@@ -312,7 +312,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Mage_Targeting" displayName="Mage_Targeting" ref="A1:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="Mage_Targeting" displayName="Mage_Targeting" ref="A1:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="지점 선택"/>
@@ -747,124 +747,106 @@
     </x:row>
     <x:row r="8" ht="70" customHeight="1">
       <x:c r="A8" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>Sanctuary</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="str">
+        <x:v>회복의 성역</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>생존 지원</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
-        <x:v>GaleBlades</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="str">
-        <x:v>질풍 칼날</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="str">
-        <x:v>관통 파동</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="F8" s="9" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G8" s="9" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="H8" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I8" s="5" t="str">
-        <x:v>바람 칼날이 일직선으로 날아가 경로상의 적을 관통합니다.</x:v>
+        <x:v>성역을 펼쳐 범위 안에서 체력 비율이 가장 낮은 왕국군을 반복해서 회복합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="70" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>Sanctuary</x:v>
+        <x:v>Meteor</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>회복의 성역</x:v>
+        <x:v>운석 낙하</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>생존 지원</x:v>
+        <x:v>예고 폭발</x:v>
       </x:c>
       <x:c r="E9" s="9" t="n">
-        <x:v>45</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="F9" s="9" t="n">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G9" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="H9" s="9" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="I9" s="5" t="str">
-        <x:v>성역을 펼쳐 범위 안에서 체력 비율이 가장 낮은 왕국군을 반복해서 회복합니다.</x:v>
+        <x:v>운석을 떨어뜨려 주변 적을 공격합니다. 착탄 지점의 잔열이 두 번 더 피해를 줍니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="70" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>Meteor</x:v>
+        <x:v>VoidRift</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>운석 낙하</x:v>
+        <x:v>공허 균열</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>예고 폭발</x:v>
+        <x:v>흡인과 붕괴</x:v>
       </x:c>
       <x:c r="E10" s="9" t="n">
-        <x:v>260</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F10" s="9" t="n">
-        <x:v>16</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G10" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H10" s="9" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
-        <x:v>운석을 떨어뜨려 주변 적을 공격합니다. 남은 불길이 두 번 더 피해를 줍니다.</x:v>
+        <x:v>균열보다 50% 넓은 범위의 적을 끌어당깁니다. 균열 안에서 지속 피해를 주고 닫힐 때 폭발합니다. 보스는 끌어당기지 못합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="70" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>VoidRift</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="str">
-        <x:v>공허 균열</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>흡인과 붕괴</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="n">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H11" s="9" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="I11" s="5" t="str">
-        <x:v>적이 모인 곳의 허공에 원형 균열을 엽니다. 균열 안의 적을 중심으로 끌어당기며 지속 피해를 주고, 닫힐 때 폭발합니다. 보스는 끌어당기지 못합니다.</x:v>
-      </x:c>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="5"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
+      <x:c r="E11" s="9"/>
+      <x:c r="F11" s="9"/>
+      <x:c r="G11" s="9"/>
+      <x:c r="H11" s="9"/>
+      <x:c r="I11" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7912bafa8f142b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8afb544d4874fde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -984,7 +966,7 @@
       <x:c r="N2" s="5" t="str">
         <x:v>Lightning_SFX</x:v>
       </x:c>
-      <x:c r="O2" s="5" t="str"/>
+      <x:c r="O2" s="5"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="9" t="n">
@@ -1030,7 +1012,7 @@
       <x:c r="N3" s="5" t="str">
         <x:v>Ice_Spike_SFX</x:v>
       </x:c>
-      <x:c r="O3" s="5" t="str"/>
+      <x:c r="O3" s="5"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="9" t="n">
@@ -1124,7 +1106,7 @@
       <x:c r="N5" s="5" t="str">
         <x:v>Charge_Shot_SFX</x:v>
       </x:c>
-      <x:c r="O5" s="5" t="str"/>
+      <x:c r="O5" s="5"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="9" t="n">
@@ -1170,7 +1152,7 @@
       <x:c r="N6" s="5" t="str">
         <x:v>Water_Splash_SFX</x:v>
       </x:c>
-      <x:c r="O6" s="5" t="str"/>
+      <x:c r="O6" s="5"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="9" t="n">
@@ -1216,24 +1198,24 @@
       <x:c r="N7" s="5" t="str">
         <x:v>Ice_Block_SFX</x:v>
       </x:c>
-      <x:c r="O7" s="5" t="str"/>
+      <x:c r="O7" s="5"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:f>'Skills'!B8</x:f>
-        <x:v>GaleBlades</x:v>
+        <x:v>Sanctuary</x:v>
       </x:c>
       <x:c r="C8" s="18" t="n">
-        <x:v>0.550000011920929</x:v>
+        <x:v>1.899999976158142</x:v>
       </x:c>
       <x:c r="D8" s="18" t="n">
-        <x:v>0.800000011920929</x:v>
+        <x:v>4.199999809265137</x:v>
       </x:c>
       <x:c r="E8" s="18" t="n">
-        <x:v>0.4000000059604645</x:v>
+        <x:v>0.699999988079071</x:v>
       </x:c>
       <x:c r="F8" s="18" t="n">
         <x:v>0</x:v>
@@ -1245,7 +1227,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="17" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J8" s="5" t="str">
         <x:v>A4/A8 타격 수 보너스</x:v>
@@ -1260,26 +1242,26 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N8" s="5" t="str">
-        <x:v>Slash_Attack_SFX</x:v>
-      </x:c>
-      <x:c r="O8" s="5" t="str"/>
+        <x:v>Parrying_SFX</x:v>
+      </x:c>
+      <x:c r="O8" s="5"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:f>'Skills'!B9</x:f>
-        <x:v>Sanctuary</x:v>
+        <x:v>Meteor</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
-        <x:v>1.899999976158142</x:v>
+        <x:v>1.5499999523162842</x:v>
       </x:c>
       <x:c r="D9" s="18" t="n">
-        <x:v>4.199999809265137</x:v>
+        <x:v>0.800000011920929</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:v>0.699999988079071</x:v>
+        <x:v>0.800000011920929</x:v>
       </x:c>
       <x:c r="F9" s="18" t="n">
         <x:v>0</x:v>
@@ -1288,16 +1270,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="18" t="n">
+        <x:v>0.13461539149284363</x:v>
+      </x:c>
+      <x:c r="I9" s="17" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I9" s="17" t="b">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="J9" s="5" t="str">
-        <x:v>A4/A8 타격 수 보너스</x:v>
+        <x:v>충돌 1회 + 잔열 2회</x:v>
       </x:c>
       <x:c r="K9" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L9" s="9" t="n">
         <x:v>100</x:v>
@@ -1306,44 +1288,44 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N9" s="5" t="str">
-        <x:v>Parrying_SFX</x:v>
-      </x:c>
-      <x:c r="O9" s="5" t="str"/>
+        <x:v>Fire_Tornado_SFX</x:v>
+      </x:c>
+      <x:c r="O9" s="5"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:f>'Skills'!B10</x:f>
-        <x:v>Meteor</x:v>
+        <x:v>VoidRift</x:v>
       </x:c>
       <x:c r="C10" s="18" t="n">
-        <x:v>1.5499999523162842</x:v>
+        <x:v>1.2999999523162842</x:v>
       </x:c>
       <x:c r="D10" s="18" t="n">
-        <x:v>0.800000011920929</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E10" s="18" t="n">
-        <x:v>0.800000011920929</x:v>
+        <x:v>0.6000000238418579</x:v>
       </x:c>
       <x:c r="F10" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>0.8500000238418579</x:v>
       </x:c>
       <x:c r="G10" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>0.20000000298023224</x:v>
       </x:c>
       <x:c r="H10" s="18" t="n">
-        <x:v>0.13461539149284363</x:v>
+        <x:v>4.285714149475098</x:v>
       </x:c>
       <x:c r="I10" s="17" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="5" t="str">
-        <x:v>충돌 1회 + 잔불 2회</x:v>
+        <x:v>반복 피해 + 마지막 붕괴</x:v>
       </x:c>
       <x:c r="K10" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L10" s="9" t="n">
         <x:v>100</x:v>
@@ -1352,60 +1334,31 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N10" s="5" t="str">
-        <x:v>Fire_Tornado_SFX</x:v>
-      </x:c>
-      <x:c r="O10" s="5" t="str"/>
+        <x:v>Charge_Shot_SFX</x:v>
+      </x:c>
+      <x:c r="O10" s="5"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str">
-        <x:f>'Skills'!B11</x:f>
-        <x:v>VoidRift</x:v>
-      </x:c>
-      <x:c r="C11" s="18" t="n">
-        <x:v>1.2999999523162842</x:v>
-      </x:c>
-      <x:c r="D11" s="18" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E11" s="18" t="n">
-        <x:v>0.6000000238418579</x:v>
-      </x:c>
-      <x:c r="F11" s="18" t="n">
-        <x:v>0.8500000238418579</x:v>
-      </x:c>
-      <x:c r="G11" s="18" t="n">
-        <x:v>0.20000000298023224</x:v>
-      </x:c>
-      <x:c r="H11" s="18" t="n">
-        <x:v>4.285714149475098</x:v>
-      </x:c>
-      <x:c r="I11" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J11" s="5" t="str">
-        <x:v>반복 피해 + 마지막 붕괴</x:v>
-      </x:c>
-      <x:c r="K11" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L11" s="9" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="M11" s="9" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="N11" s="5" t="str">
-        <x:v>Charge_Shot_SFX</x:v>
-      </x:c>
-      <x:c r="O11" s="5" t="str"/>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="16"/>
+      <x:c r="C11" s="18"/>
+      <x:c r="D11" s="18"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18"/>
+      <x:c r="G11" s="18"/>
+      <x:c r="H11" s="18"/>
+      <x:c r="I11" s="9"/>
+      <x:c r="J11" s="5"/>
+      <x:c r="K11" s="9"/>
+      <x:c r="L11" s="9"/>
+      <x:c r="M11" s="9"/>
+      <x:c r="N11" s="5"/>
+      <x:c r="O11" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccbff2996eec4f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56ffb972778641fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1690,17 +1643,17 @@
     </x:row>
     <x:row r="8" ht="90" customHeight="1">
       <x:c r="A8" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:f>'Skills'!C8</x:f>
-        <x:v>질풍 칼날</x:v>
+        <x:v>회복의 성역</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
         <x:v>미정</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>피해량 +15%. 전용 효과는 준비 중입니다.</x:v>
+        <x:v>회복량 +15%. 전용 효과는 준비 중입니다.</x:v>
       </x:c>
       <x:c r="E8" s="9" t="n">
         <x:v>10</x:v>
@@ -1723,17 +1676,17 @@
     </x:row>
     <x:row r="9" ht="90" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:f>'Skills'!C9</x:f>
-        <x:v>회복의 성역</x:v>
+        <x:v>운석 낙하</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>미정</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>회복량 +15%. 전용 효과는 준비 중입니다.</x:v>
+        <x:v>피해량 +15%. 전용 효과는 준비 중입니다.</x:v>
       </x:c>
       <x:c r="E9" s="9" t="n">
         <x:v>10</x:v>
@@ -1756,11 +1709,11 @@
     </x:row>
     <x:row r="10" ht="90" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:f>'Skills'!C10</x:f>
-        <x:v>운석 낙하</x:v>
+        <x:v>공허 균열</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
         <x:v>미정</x:v>
@@ -1788,32 +1741,15 @@
       <x:c r="N10" s="5"/>
     </x:row>
     <x:row r="11" ht="90" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str">
-        <x:f>'Skills'!C11</x:f>
-        <x:v>공허 균열</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="str">
-        <x:v>미정</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>피해량 +15%. 전용 효과는 준비 중입니다.</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="n">
-        <x:v>1.149999976158142</x:v>
-      </x:c>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="16"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
+      <x:c r="E11" s="9"/>
+      <x:c r="F11" s="9"/>
+      <x:c r="G11" s="9"/>
       <x:c r="H11" s="5"/>
-      <x:c r="I11" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="I11" s="9"/>
       <x:c r="J11" s="5"/>
       <x:c r="K11" s="5"/>
       <x:c r="L11" s="5"/>
@@ -1823,7 +1759,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2101a43777c74708"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fdcf6085a9147f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1891,7 +1827,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D2" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E2" s="9" t="n">
         <x:v>55</x:v>
@@ -1902,18 +1838,18 @@
       </x:c>
       <x:c r="G2" s="20" t="n">
         <x:f>F2/D2</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H2" s="20" t="n">
         <x:f>(F2+1)/D2</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I2" s="20" t="n">
         <x:f>H2/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J2" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -1928,7 +1864,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D3" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E3" s="9" t="n">
         <x:v>55</x:v>
@@ -1939,18 +1875,18 @@
       </x:c>
       <x:c r="G3" s="20" t="n">
         <x:f>F3/D3</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H3" s="20" t="n">
         <x:f>(F3+1)/D3</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I3" s="20" t="n">
         <x:f>H3/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J3" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -1965,7 +1901,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D4" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E4" s="9" t="n">
         <x:v>55</x:v>
@@ -1976,18 +1912,18 @@
       </x:c>
       <x:c r="G4" s="20" t="n">
         <x:f>F4/D4</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H4" s="20" t="n">
         <x:f>(F4+1)/D4</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I4" s="20" t="n">
         <x:f>H4/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J4" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -2002,7 +1938,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D5" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:v>55</x:v>
@@ -2013,18 +1949,18 @@
       </x:c>
       <x:c r="G5" s="20" t="n">
         <x:f>F5/D5</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H5" s="20" t="n">
         <x:f>(F5+1)/D5</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I5" s="20" t="n">
         <x:f>H5/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J5" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -2039,7 +1975,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E6" s="9" t="n">
         <x:v>55</x:v>
@@ -2050,18 +1986,18 @@
       </x:c>
       <x:c r="G6" s="20" t="n">
         <x:f>F6/D6</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H6" s="20" t="n">
         <x:f>(F6+1)/D6</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I6" s="20" t="n">
         <x:f>H6/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J6" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -2076,7 +2012,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D7" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
         <x:v>55</x:v>
@@ -2087,33 +2023,33 @@
       </x:c>
       <x:c r="G7" s="20" t="n">
         <x:f>F7/D7</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H7" s="20" t="n">
         <x:f>(F7+1)/D7</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I7" s="20" t="n">
         <x:f>H7/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J7" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:f>'Skills'!C8</x:f>
-        <x:v>질풍 칼날</x:v>
+        <x:v>회복의 성역</x:v>
       </x:c>
       <x:c r="C8" s="9" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D8" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E8" s="9" t="n">
         <x:v>55</x:v>
@@ -2124,33 +2060,33 @@
       </x:c>
       <x:c r="G8" s="20" t="n">
         <x:f>F8/D8</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H8" s="20" t="n">
         <x:f>(F8+1)/D8</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I8" s="20" t="n">
         <x:f>H8/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J8" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:f>'Skills'!C9</x:f>
-        <x:v>회복의 성역</x:v>
+        <x:v>운석 낙하</x:v>
       </x:c>
       <x:c r="C9" s="9" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D9" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E9" s="9" t="n">
         <x:v>55</x:v>
@@ -2161,33 +2097,33 @@
       </x:c>
       <x:c r="G9" s="20" t="n">
         <x:f>F9/D9</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H9" s="20" t="n">
         <x:f>(F9+1)/D9</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I9" s="20" t="n">
         <x:f>H9/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J9" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:f>'Skills'!C10</x:f>
-        <x:v>운석 낙하</x:v>
+        <x:v>공허 균열</x:v>
       </x:c>
       <x:c r="C10" s="9" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D10" s="19" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.05555555555555555</x:v>
       </x:c>
       <x:c r="E10" s="9" t="n">
         <x:v>55</x:v>
@@ -2198,61 +2134,36 @@
       </x:c>
       <x:c r="G10" s="20" t="n">
         <x:f>F10/D10</x:f>
-        <x:v>40</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="H10" s="20" t="n">
         <x:f>(F10+1)/D10</x:f>
-        <x:v>60</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I10" s="20" t="n">
         <x:f>H10/21</x:f>
-        <x:v>2.857142857142857</x:v>
+        <x:v>2.5714285714285716</x:v>
       </x:c>
       <x:c r="J10" s="9" t="n">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str">
-        <x:f>'Skills'!C11</x:f>
-        <x:v>공허 균열</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="D11" s="19" t="n">
-        <x:v>0.05</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F11" s="5" t="n">
-        <x:f>ROUNDUP(E11/C11,0)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G11" s="20" t="n">
-        <x:f>F11/D11</x:f>
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="H11" s="20" t="n">
-        <x:f>(F11+1)/D11</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I11" s="20" t="n">
-        <x:f>H11/21</x:f>
-        <x:v>2.857142857142857</x:v>
-      </x:c>
-      <x:c r="J11" s="9" t="n">
-        <x:v>105</x:v>
-      </x:c>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="16"/>
+      <x:c r="C11" s="9"/>
+      <x:c r="D11" s="19"/>
+      <x:c r="E11" s="9"/>
+      <x:c r="F11" s="5"/>
+      <x:c r="G11" s="20"/>
+      <x:c r="H11" s="20"/>
+      <x:c r="I11" s="20"/>
+      <x:c r="J11" s="9"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R422a35627e2648dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf66936d1f6954a4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4508,7 +4419,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e724c77b5947fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8363c378f7ec4707"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4584,8 +4495,8 @@
       <x:c r="F2" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/Lightning.prefab</x:v>
       </x:c>
-      <x:c r="G2" s="5" t="str"/>
-      <x:c r="H2" s="5" t="str"/>
+      <x:c r="G2" s="5"/>
+      <x:c r="H2" s="5"/>
       <x:c r="I2" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/LightningBloomStrike.prefab</x:v>
       </x:c>
@@ -4613,8 +4524,8 @@
       <x:c r="F3" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/IceSpike.prefab</x:v>
       </x:c>
-      <x:c r="G3" s="5" t="str"/>
-      <x:c r="H3" s="5" t="str"/>
+      <x:c r="G3" s="5"/>
+      <x:c r="H3" s="5"/>
       <x:c r="I3" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/IceBloomCrystal.prefab</x:v>
       </x:c>
@@ -4642,10 +4553,10 @@
       <x:c r="F4" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/FireTornado.prefab</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="str"/>
-      <x:c r="H4" s="5" t="str"/>
-      <x:c r="I4" s="5" t="str"/>
-      <x:c r="J4" s="5" t="str"/>
+      <x:c r="G4" s="5"/>
+      <x:c r="H4" s="5"/>
+      <x:c r="I4" s="5"/>
+      <x:c r="J4" s="5"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="9" t="n">
@@ -4667,12 +4578,12 @@
       <x:c r="F5" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/ArcaneVolley.prefab</x:v>
       </x:c>
-      <x:c r="G5" s="5" t="str"/>
+      <x:c r="G5" s="5"/>
       <x:c r="H5" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/ArcaneImpact.prefab</x:v>
       </x:c>
-      <x:c r="I5" s="5" t="str"/>
-      <x:c r="J5" s="5" t="str"/>
+      <x:c r="I5" s="5"/>
+      <x:c r="J5" s="5"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="9" t="n">
@@ -4694,10 +4605,10 @@
       <x:c r="F6" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/VenomMist.prefab</x:v>
       </x:c>
-      <x:c r="G6" s="5" t="str"/>
-      <x:c r="H6" s="5" t="str"/>
-      <x:c r="I6" s="5" t="str"/>
-      <x:c r="J6" s="5" t="str"/>
+      <x:c r="G6" s="5"/>
+      <x:c r="H6" s="5"/>
+      <x:c r="I6" s="5"/>
+      <x:c r="J6" s="5"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="9" t="n">
@@ -4722,122 +4633,109 @@
       <x:c r="G7" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/GroundTelegraph.prefab</x:v>
       </x:c>
-      <x:c r="H7" s="5" t="str"/>
-      <x:c r="I7" s="5" t="str"/>
-      <x:c r="J7" s="5" t="str"/>
+      <x:c r="H7" s="5"/>
+      <x:c r="I7" s="5"/>
+      <x:c r="J7" s="5"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:f>'Skills'!B8</x:f>
-        <x:v>GaleBlades</x:v>
+        <x:v>Sanctuary</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>Assets/MageTower/SO/GaleBlades/MageTowerSkill_GaleBlades.asset</x:v>
+        <x:v>Assets/MageTower/SO/Sanctuary/MageTowerSkill_Sanctuary.asset</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/GaleBlades.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/Sanctuary.png</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/GaleBlades_Bloom.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/Sanctuary_Bloom.png</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/GaleBlades.prefab</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="str"/>
-      <x:c r="H8" s="5" t="str"/>
-      <x:c r="I8" s="5" t="str"/>
-      <x:c r="J8" s="5" t="str"/>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/Sanctuary.prefab</x:v>
+      </x:c>
+      <x:c r="G8" s="5"/>
+      <x:c r="H8" s="5" t="str">
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/SanctuaryHeal.prefab</x:v>
+      </x:c>
+      <x:c r="I8" s="5"/>
+      <x:c r="J8" s="5"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:f>'Skills'!B9</x:f>
-        <x:v>Sanctuary</x:v>
+        <x:v>Meteor</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>Assets/MageTower/SO/Sanctuary/MageTowerSkill_Sanctuary.asset</x:v>
+        <x:v>Assets/MageTower/SO/Meteor/MageTowerSkill_Meteor.asset</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/Sanctuary.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/Meteor.png</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/Sanctuary_Bloom.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/Meteor_Bloom.png</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/Sanctuary.prefab</x:v>
-      </x:c>
-      <x:c r="G9" s="5" t="str"/>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
+      </x:c>
+      <x:c r="G9" s="5" t="str">
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/GroundTelegraph.prefab</x:v>
+      </x:c>
       <x:c r="H9" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/SanctuaryHeal.prefab</x:v>
-      </x:c>
-      <x:c r="I9" s="5" t="str"/>
-      <x:c r="J9" s="5" t="str"/>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
+      </x:c>
+      <x:c r="I9" s="5"/>
+      <x:c r="J9" s="5"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:f>'Skills'!B10</x:f>
-        <x:v>Meteor</x:v>
+        <x:v>VoidRift</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>Assets/MageTower/SO/Meteor/MageTowerSkill_Meteor.asset</x:v>
+        <x:v>Assets/MageTower/SO/VoidRift/MageTowerSkill_VoidRift.asset</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/Meteor.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/VoidRift.png</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/Meteor_Bloom.png</x:v>
+        <x:v>Assets/_Project/Art/Icons/MageTower/VoidRift_Bloom.png</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/GroundTelegraph.prefab</x:v>
-      </x:c>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/VoidRift.prefab</x:v>
+      </x:c>
+      <x:c r="G10" s="5"/>
       <x:c r="H10" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
-      </x:c>
-      <x:c r="I10" s="5" t="str"/>
-      <x:c r="J10" s="5" t="str"/>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/VoidCollapse.prefab</x:v>
+      </x:c>
+      <x:c r="I10" s="5"/>
+      <x:c r="J10" s="5"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str">
-        <x:f>'Skills'!B11</x:f>
-        <x:v>VoidRift</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="str">
-        <x:v>Assets/MageTower/SO/VoidRift/MageTowerSkill_VoidRift.asset</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/VoidRift.png</x:v>
-      </x:c>
-      <x:c r="E11" s="5" t="str">
-        <x:v>Assets/_Project/Art/Icons/MageTower/VoidRift_Bloom.png</x:v>
-      </x:c>
-      <x:c r="F11" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/VoidRift.prefab</x:v>
-      </x:c>
-      <x:c r="G11" s="5" t="str"/>
-      <x:c r="H11" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/VoidCollapse.prefab</x:v>
-      </x:c>
-      <x:c r="I11" s="5" t="str"/>
-      <x:c r="J11" s="5" t="str"/>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="16"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
+      <x:c r="E11" s="5"/>
+      <x:c r="F11" s="5"/>
+      <x:c r="G11" s="5"/>
+      <x:c r="H11" s="5"/>
+      <x:c r="I11" s="5"/>
+      <x:c r="J11" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0294a0713b664c4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f47310ac26043f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4957,65 +4855,56 @@
     </x:row>
     <x:row r="8" ht="76" customHeight="1">
       <x:c r="A8" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>유효 표적 방향으로 관통 경로 설정</x:v>
+        <x:v>생존 아군 중 HP 비율 최저</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>파동이 실제 통과한 경로 안 최대 5체 · 파동당 같은 적 1회</x:v>
+        <x:v>매 회복마다 대상 재선정</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>단발 파동 전면</x:v>
+        <x:v>한 번 등장 후 지속시간 동안 회복 파동. 종료 시 한 번 퇴장</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
       <x:c r="A9" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>생존 아군 중 HP 비율 최저</x:v>
+        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>매 회복마다 대상 재선정</x:v>
+        <x:v>예고 위치 고정 · 충돌 후 잔열 2회</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>성역 후면 · 회복 반짝임 전면</x:v>
+        <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="76" customHeight="1">
       <x:c r="A10" s="9" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
+        <x:v>공중 균열, 피해 반경 1.3, 흡입 반경 1.95 월드 단위</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>예고 위치 고정 · 충돌 후 잔불 2회</x:v>
+        <x:v>흡입은 보이는 균열보다 50% 넓게 적용. 피해·붕괴 반경 유지</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>운석과 폭발 전면 · 잔불 후면</x:v>
+        <x:v>지속 균열 후면 · 붕괴 전면</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="76" customHeight="1">
-      <x:c r="A11" s="9" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="str">
-        <x:v>허공 원 안 몸체 중심만 흡인 · 보스 흡인 면역
-약한 감속으로 기존 강한 감속을 덮어쓰지 않음</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>지속 균열 후면 · 붕괴 전면</x:v>
-      </x:c>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="5"/>
+      <x:c r="C11" s="5"/>
+      <x:c r="D11" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f77bf989dcb433c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3f445c770e24027"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5076,7 +4965,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.10.2 · 스킬 데이터 계약 mage-3 · 스킬 ID 0~9와 기존 에셋 GUID를 유지합니다.</x:v>
+        <x:v>게임 0.12.0. 스킬 데이터 계약 mage-4. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -5092,7 +4981,7 @@
         <x:v>공통 성장</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>직접 강화 E는 비전 지식으로 0~100, 각성 A는 동일 스킬 파편으로 0~10. A4/A8에 각각 1회 추가(화염 회오리는 2틱), A마다 효과량 +5%와 쿨타임 -2%. 운석은 고정 1회 충돌과 잔불 2회이며 타격 수 보너스를 사용하지 않습니다.</x:v>
+        <x:v>직접 강화 E는 비전 지식으로 0~100, 각성 A는 동일 스킬 파편으로 0~10. A4/A8에 각각 1회 추가(화염 회오리는 2틱), A마다 효과량 +5%와 쿨타임 -2%. 운석은 고정 1회 충돌과 잔열 2회이며 타격 수 보너스를 사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
@@ -5116,7 +5005,7 @@
         <x:v>확률</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>전체 뽑기는 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 스킬 10종은 등급 없이 각각 5%로 획득합니다. 희귀도는 장비에만 적용합니다.</x:v>
+        <x:v>전체 뽑기는 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 9종 스킬은 같은 확률(각 50%/9)입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -5132,7 +5021,7 @@
         <x:v>투자 기간</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>각성 누적55파편 기준입니다. 주당21회 전부 마탑에 사용하고 최초 보상·기존 파편을 제외하면 미보유 특정 스킬의 평균 개화 기간은 60회 뽑기, 약2.86주입니다. 장비 뽑기에 주화를 나누면 더 오래 걸립니다.</x:v>
+        <x:v>각성 누적 55파편. 주당 21회 마탑 뽑기 기준으로 미보유 특정 스킬의 평균 개화 기간은 54회, 약 2.57주입니다. 기존 파편과 최초 보상은 제외합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
@@ -5140,7 +5029,7 @@
         <x:v>확률 편차</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>Acquisition의 P90은 해당 횟수까지 약90%가 목표를 달성한다는 정확한 음이항 계산입니다. 스킬당105회(약5주). 천장과 기간 보장은 없으며 수 주는 평균 목표입니다.</x:v>
+        <x:v>Acquisition의 P90은 정확한 음이항 계산입니다. 스킬당 95회까지 약 90%가 목표를 달성합니다. 천장이나 기간 보장은 없습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5172,7 +5061,7 @@
         <x:v>타격 연출</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>타격 시점에 피해·피격 반응·효과음을 맞춥니다. 별빛은 겹쳐 낙하하고 운석은 충돌 후 잔불을 남깁니다. 기절과 감속은 독립 만료하며 감속은 합산하지 않고 가장 강한 효과만 적용합니다. 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
+        <x:v>타격 시점에 피해·피격 반응·효과음을 맞춥니다. 별빛은 겹쳐 낙하하고 운석은 충돌 후 잔열을 남깁니다. 기절과 감속은 독립 만료하며 감속은 합산하지 않고 가장 강한 효과만 적용합니다. 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5204,13 +5093,13 @@
         <x:v>보류 개화</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>천벌·만년빙정 외 8종은 개화 미정으로 표기합니다. 현재는 기존 피해 또는 회복의15% 증가만 적용하며 확정된 고유 개화로 오해하지 않도록 유지합니다.</x:v>
+        <x:v>천벌·만년빙정 외 7종은 개화 미정이며 피해 또는 회복량이 15% 증가합니다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774af23012b741fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865e0bac42044ae0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(gameplay): synchronize operating plans and record restored-account b53 validation
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rd3e087a157ec40d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R81dbcc681f6a44d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R6149853889ba41a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R9ab34a80bdb54e67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="Re554c98a7e904d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R324efd102463456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rd777cf03eb074eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R076e2cb4d77c4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R5e66305b0bcb496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rb07b744bbd4642af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R776d650675f2476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R401851261137418d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R3b65024a75cd4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rbf1994a6156043d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rbfaf17bb1c8b4f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R03c33789bfde4450"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="202" formatCode="0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,6 +60,10 @@
       <x:color rgb="FF206447"/>
       <x:name val="Malgun Gothic"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -80,7 +84,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -172,6 +176,10 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -672,13 +680,13 @@
         <x:v>전장 낙하</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
-        <x:v>62</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H5" s="9" t="n">
         <x:v>1</x:v>
@@ -742,7 +750,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="I7" s="5" t="str">
-        <x:v>바위를 연속으로 솟아올려 주변 적을 공격하고 1초간 기절시킵니다.</x:v>
+        <x:v>바위를 연속으로 솟아올려 주변 적을 공격하고 1.4초간 기절시킵니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="70" customHeight="1">
@@ -846,7 +854,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8afb544d4874fde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bd5c94c2e05400c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1074,10 +1082,10 @@
         <x:v>0.550000011920929</x:v>
       </x:c>
       <x:c r="D5" s="18" t="n">
-        <x:v>1.3199999332427979</x:v>
+        <x:v>2.16</x:v>
       </x:c>
       <x:c r="E5" s="18" t="n">
-        <x:v>0.2199999988079071</x:v>
+        <x:v>0.12</x:v>
       </x:c>
       <x:c r="F5" s="18" t="n">
         <x:v>0</x:v>
@@ -1172,7 +1180,7 @@
         <x:v>0.44999998807907104</x:v>
       </x:c>
       <x:c r="F7" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="G7" s="18" t="n">
         <x:v>0</x:v>
@@ -1209,7 +1217,7 @@
         <x:v>Sanctuary</x:v>
       </x:c>
       <x:c r="C8" s="18" t="n">
-        <x:v>1.899999976158142</x:v>
+        <x:v>2.6</x:v>
       </x:c>
       <x:c r="D8" s="18" t="n">
         <x:v>4.199999809265137</x:v>
@@ -1358,7 +1366,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56ffb972778641fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64be8cc0f0d948c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1482,7 +1490,7 @@
       </x:c>
       <x:c r="D3" s="5" t="str">
         <x:v>여러 적: 송곳 8개를 두 번 생성합니다. 각각 피해 50%.
-적 하나: 거대 빙정으로 피해 650%와 기절 2초를 줍니다.</x:v>
+적 하나: 거대 빙정으로 피해 650%를 줍니다. 기절 효과는 없습니다.</x:v>
       </x:c>
       <x:c r="E3" s="9" t="n">
         <x:v>10</x:v>
@@ -1497,7 +1505,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I3" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J3" s="5"/>
       <x:c r="K3" s="9" t="n">
@@ -1759,7 +1767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fdcf6085a9147f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca17e19059f4c6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2163,7 +2171,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf66936d1f6954a4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45dc047724e94985"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4419,7 +4427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8363c378f7ec4707"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51c64b05cc414188"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4684,9 +4692,7 @@
       <x:c r="F9" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
       </x:c>
-      <x:c r="G9" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/GroundTelegraph.prefab</x:v>
-      </x:c>
+      <x:c r="G9" s="5" t="str"/>
       <x:c r="H9" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
       </x:c>
@@ -4735,7 +4741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f47310ac26043f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefa5d3d3c134401"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4819,7 +4825,7 @@
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>별빛은 비행 전반 70% 동안 대상을 추적한 뒤 낙하 지점을 확정
-0.22초 간격 · 비행 0.48초</x:v>
+0.12초 간격 · 18개 기본 낙하 · 비행 0.48초</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
         <x:v>낙하와 충돌 전면</x:v>
@@ -4875,7 +4881,7 @@
         <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>예고 위치 고정 · 충돌 후 잔열 2회</x:v>
+        <x:v>착탄 지점 고정 · 시전 마법진 없음 · 충돌 후 잔열 2회</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
@@ -4904,7 +4910,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3f445c770e24027"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd15e8e26437e457a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4965,7 +4971,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.12.0. 스킬 데이터 계약 mage-4. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
+        <x:v>게임 0.13.0 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -5069,7 +5075,7 @@
         <x:v>외부 원본</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>ExternalAssets는 원본 저장소이며 직접 변경하지 않습니다. Assets 탭의 작업본만 사용합니다. 생성 출처는 AI/comfyui/mage-skills/20260915, 20260916-combat 및 20260917-polish입니다. 운석 잔흔은 두 모델 비교 후 채택한 단일 64px·6색 지면 데칼입니다.</x:v>
+        <x:v>ExternalAssets 원본은 보존합니다. 최신 제작은 AI/comfyui/mage-vfx/revision1~4 및 finish-manifest.json에 실제 API·UI 그래프·원본·채택/기각·비용을 기록했습니다. 운석 시전 원과 지속 불길을 제거하고 크레이터를 축소했습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -5096,10 +5102,58 @@
         <x:v>천벌·만년빙정 외 7종은 개화 미정이며 피해 또는 회복량이 15% 증가합니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="68" customHeight="1">
+      <x:c r="A23" s="24" t="str">
+        <x:v>왕국군 공격 계수</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>시전당 1회 효과량 = round(기본 효과량×1.04^E×(1+0.05A)) + round(출전 3인 ATK 합×기본 효과량/400×(1+0.005E+0.025A)). 사망한 출전 병사도 합산하고 시전 시작 시 고정합니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="68" customHeight="1">
+      <x:c r="A24" s="24" t="str">
+        <x:v>수동 시전</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>자동 OFF에서 우측 스테이지 표시 위에 장착 스킬을 나열합니다. ON이면 대응하는 퇴장 애니메이션. 준비 점등·시계 방향 쿨다운 음영·남은 초를 표시합니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="68" customHeight="1">
+      <x:c r="A25" s="24" t="str">
+        <x:v>조준 구도</x:v>
+      </x:c>
+      <x:c r="B25" s="24" t="str">
+        <x:v>발 위치 기준 원형 게임 판정과 쿼터뷰 타원 장판 표시를 구분합니다. 분산 스킬인 얼음 송곳·유성우는 드래그 시전과 쿨다운 소비를 하지 않습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="68" customHeight="1">
+      <x:c r="A26" s="24" t="str">
+        <x:v>각성 안내</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>A4/A8 추가 타격·틱, 다음 각성의 효과량·쿨타임·타격 수, A10 개화 효과를 상세 화면에 표시합니다. 운석은 추가 타격 보너스가 없습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="68" customHeight="1">
+      <x:c r="A27" s="24" t="str">
+        <x:v>성역 연출</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>반경 2.6. 한 번 상승한 불투명 문양을 유지하며 발밑 지면 파동으로 회복하고 종료 때 한 번 하강합니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="68" customHeight="1">
+      <x:c r="A28" s="24" t="str">
+        <x:v>픽셀과 레이어</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>핵심 VFX 목표 32px/월드 단위, 4~6색·Point·ASTC4×4. 단발 타격은 전면, 독 늪·잔열·흡인 등 지속 장판은 후면입니다. 이펙트가 큰 경우 원본 논리 해상도도 함께 높입니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865e0bac42044ae0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R694d7a683991474e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify spell animation polish on Android and record 0.13.1
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R5e66305b0bcb496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="Rb07b744bbd4642af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R776d650675f2476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R401851261137418d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R3b65024a75cd4b4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rbf1994a6156043d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rbfaf17bb1c8b4f4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R03c33789bfde4450"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rfb40bf9e195d4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R03eb3efe38804895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R40cd25fdcdf5449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R7b457e33fc184ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R8ac5e82532b24e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rfb662544e7264b58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R1a380916625e4f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R4a0f847c16894ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -605,7 +605,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="I2" s="5" t="str">
-        <x:v>같은 지점에 번개를 연속으로 내려 주변 적을 공격합니다.</x:v>
+        <x:v>번개를 3회 연속으로 내립니다. 4·8각성마다 같은 패턴의 낙뢰가 1회 추가됩니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="70" customHeight="1">
@@ -854,7 +854,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bd5c94c2e05400c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R833b7bd22e084c3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -942,10 +942,10 @@
         <x:v>0.550000011920929</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
-        <x:v>0.9000000357627869</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="E2" s="18" t="n">
-        <x:v>0.30000001192092896</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
         <x:v>0</x:v>
@@ -1366,7 +1366,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64be8cc0f0d948c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7174bf87fcb45a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1767,7 +1767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ca17e19059f4c6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8ffd66f2c145d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2171,7 +2171,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45dc047724e94985"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55175084dd364b3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4427,7 +4427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51c64b05cc414188"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e3fe0e4ef14420"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4741,7 +4741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefa5d3d3c134401"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref7ef47ec0f942df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4781,8 +4781,8 @@
         <x:v>적이 가장 많이 모인 지점</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>고정 원형 범위 · 천벌의 구름 높이와 벼락 길이는 상단 여백에 맞춤
-연출 높이 보정으로 타격 지점을 아래로 이동하지 않음</x:v>
+        <x:v>일반: 첫 중심 이후 0.8 이내 분산, 낙뢰마다 반경 0.55. 조준 반경 1.35.
+약 0.167초 간격으로 기본 3회, A4 4회, A8 이상 5회. 천벌 연출 유지.</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
         <x:v>즉발 낙뢰 전면 · 구름 전면</x:v>
@@ -4881,7 +4881,8 @@
         <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>착탄 지점 고정 · 시전 마법진 없음 · 충돌 후 잔열 2회</x:v>
+        <x:v>착탄 지점 고정. 시전 마법진 없음.
+2.4초 가속 낙하, 접촉 후 0.09초에 피해. 잔열 2회.</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
@@ -4910,7 +4911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd15e8e26437e457a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb70d5060c364185"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4971,7 +4972,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.13.0 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
+        <x:v>게임 0.13.1 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -5075,7 +5076,7 @@
         <x:v>외부 원본</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>ExternalAssets 원본은 보존합니다. 최신 제작은 AI/comfyui/mage-vfx/revision1~4 및 finish-manifest.json에 실제 API·UI 그래프·원본·채택/기각·비용을 기록했습니다. 운석 시전 원과 지속 불길을 제거하고 크레이터를 축소했습니다.</x:v>
+        <x:v>ExternalAssets 원본은 보존합니다. 제작 출처: AI/comfyui/mage-vfx/revision1~5. 일반 라이트닝은 최초 ThunderEffects 원화 복원. 운석은 Comfy 표면 마스터를 회전·화염 흐름·파편 48프레임으로 가공했습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -5153,7 +5154,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R694d7a683991474e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2372c9049dec47d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Set meteor flight to 1.5 seconds and retime animation
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rfb40bf9e195d4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R03eb3efe38804895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R40cd25fdcdf5449d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R7b457e33fc184ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R8ac5e82532b24e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rfb662544e7264b58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R1a380916625e4f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R4a0f847c16894ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rc98ca8b488ab43a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R62aef14d353e4d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="Rb654bd1f2e1a45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R1af024dc59e64e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R375048e3161446f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rcfbc5a9b1bad4e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R185f5fb4a3294e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R3011c7e3fdc546e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -854,7 +854,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R833b7bd22e084c3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38de710b36ea451d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1366,7 +1366,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7174bf87fcb45a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79950523d99c4e5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1767,7 +1767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8ffd66f2c145d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R805d4a9ac9714224"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2171,7 +2171,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55175084dd364b3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reff2ded0646a4476"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4427,7 +4427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e3fe0e4ef14420"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0139623cfc134fdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4741,7 +4741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref7ef47ec0f942df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5af9039f4114504"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4882,7 +4882,7 @@
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>착탄 지점 고정. 시전 마법진 없음.
-2.4초 가속 낙하, 접촉 후 0.09초에 피해. 잔열 2회.</x:v>
+1.5초 가속 낙하, 접촉 후 0.09초에 피해. 잔열 2회.</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
@@ -4911,7 +4911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb70d5060c364185"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe0ed84f3b1414b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4972,7 +4972,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.13.1 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
+        <x:v>게임 0.13.2 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -5154,7 +5154,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2372c9049dec47d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re36db18132344b88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Merge meteor into starfall bloom and restore impact feedback
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="Rc98ca8b488ab43a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R62aef14d353e4d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="Rb654bd1f2e1a45ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R1af024dc59e64e53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R375048e3161446f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rcfbc5a9b1bad4e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R185f5fb4a3294e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R3011c7e3fdc546e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R2b25563ab4234517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R252594dbfc684dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R9949f6ace02f4682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R55d581f3c3644ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R0397ae5074cf4a68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rdcad8e5da80041fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rf4e5a5af546e4974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rbdb279aa60c54caf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="202" formatCode="0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,13 @@
       <x:sz val="11"/>
       <x:name val="맑은 고딕"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF6B7280"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -77,6 +82,11 @@
         <x:fgColor rgb="FF253E52"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5E7EB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -84,7 +94,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -180,6 +190,55 @@
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -605,7 +664,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="I2" s="5" t="str">
-        <x:v>번개를 3회 연속으로 내립니다. 4·8각성마다 같은 패턴의 낙뢰가 1회 추가됩니다.</x:v>
+        <x:v>번개를 3회 연속으로 내립니다. 4·8각성마다 같은 패턴의 낙뢰가 1회 추가됩니다. 낙뢰 위치는 서로 간격을 두고 분산됩니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="70" customHeight="1">
@@ -677,7 +736,7 @@
         <x:v>유성우</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>전장 낙하</x:v>
+        <x:v>무작위 소범위 폭격</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:v>28</x:v>
@@ -689,10 +748,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="H5" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
-        <x:v>전장 곳곳의 적에게 별빛을 차례로 떨어뜨립니다. 별빛이 닿은 적에게 피해를 줍니다.</x:v>
+        <x:v>성역보다 조금 넓은 범위의 무작위 지점에 붉은 별빛을 떨어뜨립니다. 적을 추적하지 않으며 작은 착탄 파동 안에 범위 피해를 줍니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="70" customHeight="1">
@@ -783,32 +842,32 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="70" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
+      <x:c r="B9" s="28" t="str">
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>운석 낙하</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
-        <x:v>예고 폭발</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="n">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H9" s="9" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="I9" s="5" t="str">
-        <x:v>운석을 떨어뜨려 주변 적을 공격합니다. 착탄 지점의 잔열이 두 번 더 피해를 줍니다.</x:v>
+      <x:c r="C9" s="28" t="str">
+        <x:v>독립 운석 삭제</x:v>
+      </x:c>
+      <x:c r="D9" s="28" t="str">
+        <x:v>ID 3 개화로 통합</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="28" t="str">
+        <x:v>ID 8은 비활성 보존 ID입니다. 로스터·장착·뽑기에 나오지 않으며 유성우의 개화 메테오로 통합했습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="70" customHeight="1">
@@ -854,7 +913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38de710b36ea451d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36a81b40f5f3428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1255,50 +1314,50 @@
       <x:c r="O8" s="5"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
+      <x:c r="B9" s="28" t="str">
         <x:f>'Skills'!B9</x:f>
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="18" t="n">
+      <x:c r="C9" s="32" t="n">
         <x:v>1.5499999523162842</x:v>
       </x:c>
-      <x:c r="D9" s="18" t="n">
+      <x:c r="D9" s="32" t="n">
         <x:v>0.800000011920929</x:v>
       </x:c>
-      <x:c r="E9" s="18" t="n">
+      <x:c r="E9" s="32" t="n">
         <x:v>0.800000011920929</x:v>
       </x:c>
-      <x:c r="F9" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="18" t="n">
+      <x:c r="F9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="32" t="n">
         <x:v>0.13461539149284363</x:v>
       </x:c>
-      <x:c r="I9" s="17" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="5" t="str">
+      <x:c r="I9" s="33" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="28" t="str">
         <x:v>충돌 1회 + 잔열 2회</x:v>
       </x:c>
-      <x:c r="K9" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L9" s="9" t="n">
+      <x:c r="K9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="27" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="M9" s="9" t="n">
+      <x:c r="M9" s="27" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="N9" s="5" t="str">
+      <x:c r="N9" s="28" t="str">
         <x:v>Fire_Tornado_SFX</x:v>
       </x:c>
-      <x:c r="O9" s="5"/>
+      <x:c r="O9" s="28"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -1366,7 +1425,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79950523d99c4e5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a404bc63e948f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1417,7 +1476,7 @@
         <x:v>PowerMultiplier</x:v>
       </x:c>
       <x:c r="H1" s="8" t="str">
-        <x:v>CrowdPerHitMultiplier</x:v>
+        <x:v>CrowdOrFieldTickMultiplier</x:v>
       </x:c>
       <x:c r="I1" s="8" t="str">
         <x:v>SingleTargetStunSec</x:v>
@@ -1550,7 +1609,7 @@
       <x:c r="M4" s="5"/>
       <x:c r="N4" s="5"/>
     </x:row>
-    <x:row r="5" ht="90" customHeight="1">
+    <x:row r="5" ht="110" customHeight="1">
       <x:c r="A5" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1559,29 +1618,39 @@
         <x:v>유성우</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>미정</x:v>
+        <x:v>메테오</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>피해량 +15%. 전용 효과는 준비 중입니다.</x:v>
+        <x:v>거대한 운석이 1.5초 낙하해 피해 2000%를 줍니다.
+균열 장판이 3.5초 동안 0.5초마다 피해 200%를 주고, 안의 적을 60% 감속합니다.
+쿨타임 1.6배. 장판 밖에서는 약 0.12초 안에 감속이 해제되고 더 약한 기존 감속이 복구됩니다.</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>1.6</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
-        <x:v>1.149999976158142</x:v>
-      </x:c>
-      <x:c r="H5" s="5"/>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I5" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J5" s="5"/>
+      <x:c r="J5" s="5" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="K5" s="5"/>
       <x:c r="L5" s="5"/>
-      <x:c r="M5" s="5"/>
-      <x:c r="N5" s="5"/>
+      <x:c r="M5" s="5" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="N5" s="5" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="90" customHeight="1">
       <x:c r="A6" s="9" t="n">
@@ -1683,37 +1752,37 @@
       <x:c r="N8" s="5"/>
     </x:row>
     <x:row r="9" ht="90" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
+      <x:c r="B9" s="28" t="str">
         <x:f>'Skills'!C9</x:f>
-        <x:v>운석 낙하</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>미정</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
-        <x:v>피해량 +15%. 전용 효과는 준비 중입니다.</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="n">
+        <x:v>독립 운석 삭제</x:v>
+      </x:c>
+      <x:c r="C9" s="28" t="str">
+        <x:v>통합됨</x:v>
+      </x:c>
+      <x:c r="D9" s="28" t="str">
+        <x:v>ID 3 메테오 개화 항목을 사용합니다.</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F9" s="9" t="n">
+      <x:c r="F9" s="27" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G9" s="9" t="n">
+      <x:c r="G9" s="27" t="n">
         <x:v>1.149999976158142</x:v>
       </x:c>
-      <x:c r="H9" s="5"/>
-      <x:c r="I9" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="5"/>
-      <x:c r="K9" s="5"/>
-      <x:c r="L9" s="5"/>
-      <x:c r="M9" s="5"/>
-      <x:c r="N9" s="5"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="28"/>
+      <x:c r="K9" s="28"/>
+      <x:c r="L9" s="28"/>
+      <x:c r="M9" s="28"/>
+      <x:c r="N9" s="28"/>
     </x:row>
     <x:row r="10" ht="90" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -1767,7 +1836,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R805d4a9ac9714224"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f09b68380e4338"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1835,7 +1904,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D2" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E2" s="9" t="n">
         <x:v>55</x:v>
@@ -1846,18 +1915,18 @@
       </x:c>
       <x:c r="G2" s="20" t="n">
         <x:f>F2/D2</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H2" s="20" t="n">
         <x:f>(F2+1)/D2</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I2" s="20" t="n">
         <x:f>H2/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J2" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -1872,7 +1941,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D3" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E3" s="9" t="n">
         <x:v>55</x:v>
@@ -1883,18 +1952,18 @@
       </x:c>
       <x:c r="G3" s="20" t="n">
         <x:f>F3/D3</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H3" s="20" t="n">
         <x:f>(F3+1)/D3</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I3" s="20" t="n">
         <x:f>H3/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J3" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -1909,7 +1978,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D4" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E4" s="9" t="n">
         <x:v>55</x:v>
@@ -1920,18 +1989,18 @@
       </x:c>
       <x:c r="G4" s="20" t="n">
         <x:f>F4/D4</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H4" s="20" t="n">
         <x:f>(F4+1)/D4</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I4" s="20" t="n">
         <x:f>H4/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J4" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
@@ -1946,7 +2015,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D5" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:v>55</x:v>
@@ -1957,18 +2026,18 @@
       </x:c>
       <x:c r="G5" s="20" t="n">
         <x:f>F5/D5</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H5" s="20" t="n">
         <x:f>(F5+1)/D5</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I5" s="20" t="n">
         <x:f>H5/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J5" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -1983,7 +2052,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E6" s="9" t="n">
         <x:v>55</x:v>
@@ -1994,18 +2063,18 @@
       </x:c>
       <x:c r="G6" s="20" t="n">
         <x:f>F6/D6</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H6" s="20" t="n">
         <x:f>(F6+1)/D6</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I6" s="20" t="n">
         <x:f>H6/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J6" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -2020,7 +2089,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D7" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
         <x:v>55</x:v>
@@ -2031,18 +2100,18 @@
       </x:c>
       <x:c r="G7" s="20" t="n">
         <x:f>F7/D7</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H7" s="20" t="n">
         <x:f>(F7+1)/D7</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I7" s="20" t="n">
         <x:f>H7/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J7" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -2057,7 +2126,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D8" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E8" s="9" t="n">
         <x:v>55</x:v>
@@ -2068,55 +2137,51 @@
       </x:c>
       <x:c r="G8" s="20" t="n">
         <x:f>F8/D8</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H8" s="20" t="n">
         <x:f>(F8+1)/D8</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I8" s="20" t="n">
         <x:f>H8/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J8" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
+      <x:c r="B9" s="28" t="str">
         <x:f>'Skills'!C9</x:f>
-        <x:v>운석 낙하</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="D9" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F9" s="5" t="n">
-        <x:f>ROUNDUP(E9/C9,0)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G9" s="20" t="n">
-        <x:f>F9/D9</x:f>
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="H9" s="20" t="n">
-        <x:f>(F9+1)/D9</x:f>
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="I9" s="20" t="n">
-        <x:f>H9/21</x:f>
-        <x:v>2.5714285714285716</x:v>
-      </x:c>
-      <x:c r="J9" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>독립 운석 삭제</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="28" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="27" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -2131,7 +2196,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="D10" s="19" t="n">
-        <x:v>0.05555555555555555</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="E10" s="9" t="n">
         <x:v>55</x:v>
@@ -2142,18 +2207,18 @@
       </x:c>
       <x:c r="G10" s="20" t="n">
         <x:f>F10/D10</x:f>
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H10" s="20" t="n">
         <x:f>(F10+1)/D10</x:f>
-        <x:v>54</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I10" s="20" t="n">
         <x:f>H10/21</x:f>
-        <x:v>2.5714285714285716</x:v>
+        <x:v>2.2857142857142856</x:v>
       </x:c>
       <x:c r="J10" s="9" t="n">
-        <x:v>95</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -2171,7 +2236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reff2ded0646a4476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e7c2d7649541c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4427,7 +4492,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0139623cfc134fdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e861d794534565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4449,6 +4514,7 @@
     <x:col min="8" max="8" width="86" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="86" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="88" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="88" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="46" customHeight="1">
@@ -4482,6 +4548,9 @@
       <x:c r="J1" s="8" t="str">
         <x:v>BloomCastingPrefabPath</x:v>
       </x:c>
+      <x:c r="K1" t="str">
+        <x:v>BloomSecondaryPrefabPath</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="9" t="n">
@@ -4511,6 +4580,7 @@
       <x:c r="J2" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/LightningBloomCloud.prefab</x:v>
       </x:c>
+      <x:c r="K2" t="str"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="9" t="n">
@@ -4540,6 +4610,7 @@
       <x:c r="J3" s="5" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/IceBloomWarning.prefab</x:v>
       </x:c>
+      <x:c r="K3" t="str"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="9" t="n">
@@ -4565,6 +4636,7 @@
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5"/>
       <x:c r="J4" s="5"/>
+      <x:c r="K4" t="str"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="9" t="n">
@@ -4588,10 +4660,15 @@
       </x:c>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5" t="str">
-        <x:v>Assets/_Project/Prefabs/VFX/MageTower/ArcaneImpact.prefab</x:v>
-      </x:c>
-      <x:c r="I5" s="5"/>
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/StarfallPulse.prefab</x:v>
+      </x:c>
+      <x:c r="I5" s="5" t="str">
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
+      </x:c>
       <x:c r="J5" s="5"/>
+      <x:c r="K5" t="str">
+        <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="9" t="n">
@@ -4617,6 +4694,7 @@
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5"/>
       <x:c r="J6" s="5"/>
+      <x:c r="K6" t="str"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="9" t="n">
@@ -4644,6 +4722,7 @@
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
+      <x:c r="K7" t="str"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="9" t="n">
@@ -4671,33 +4750,35 @@
       </x:c>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>
+      <x:c r="K8" t="str"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="16" t="str">
+      <x:c r="B9" s="28" t="str">
         <x:f>'Skills'!B9</x:f>
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="str">
+      <x:c r="C9" s="28" t="str">
         <x:v>Assets/MageTower/SO/Meteor/MageTowerSkill_Meteor.asset</x:v>
       </x:c>
-      <x:c r="D9" s="5" t="str">
+      <x:c r="D9" s="28" t="str">
         <x:v>Assets/_Project/Art/Icons/MageTower/Meteor.png</x:v>
       </x:c>
-      <x:c r="E9" s="5" t="str">
+      <x:c r="E9" s="28" t="str">
         <x:v>Assets/_Project/Art/Icons/MageTower/Meteor_Bloom.png</x:v>
       </x:c>
-      <x:c r="F9" s="5" t="str">
+      <x:c r="F9" s="28" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
       </x:c>
-      <x:c r="G9" s="5" t="str"/>
-      <x:c r="H9" s="5" t="str">
+      <x:c r="G9" s="28" t="str"/>
+      <x:c r="H9" s="28" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
       </x:c>
-      <x:c r="I9" s="5"/>
-      <x:c r="J9" s="5"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="28"/>
+      <x:c r="K9" t="str"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -4725,6 +4806,7 @@
       </x:c>
       <x:c r="I10" s="5"/>
       <x:c r="J10" s="5"/>
+      <x:c r="K10" t="str"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="9"/>
@@ -4741,7 +4823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5af9039f4114504"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ec304716b734fa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4781,8 +4863,8 @@
         <x:v>적이 가장 많이 모인 지점</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>일반: 첫 중심 이후 0.8 이내 분산, 낙뢰마다 반경 0.55. 조준 반경 1.35.
-약 0.167초 간격으로 기본 3회, A4 4회, A8 이상 5회. 천벌 연출 유지.</x:v>
+        <x:v>일반: 첫 중심 이후 1.15 이내 분산, 기존 낙뢰와 0.45 이상 간격을 우선 확보. 낙뢰마다 반경 0.55, 조준 반경 1.7.
+약 0.167초 간격으로 A0 3회, A4 4회, A8 5회. 매 타격 약한 흔들림, 천벌 타격 때 강한 흔들림.</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
         <x:v>즉발 낙뢰 전면 · 구름 전면</x:v>
@@ -4816,19 +4898,21 @@
         <x:v>지속 장판 후면</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="76" customHeight="1">
+    <x:row r="5" ht="145" customHeight="1">
       <x:c r="A5" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>전장 내 적을 차례로 선택</x:v>
+        <x:v>전장 중심의 고정 타원 범위 · 적을 지정하거나 추적하지 않음</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>별빛은 비행 전반 70% 동안 대상을 추적한 뒤 낙하 지점을 확정
-0.12초 간격 · 18개 기본 낙하 · 비행 0.48초</x:v>
+        <x:v>기본: 반경 3, Y축 0.65배 타원 안 균등 난수. 18개/A4 19개/A8 20개, 0.12초 간격, 비행 0.48초.
+착탄 파동 반경 0.55(Y 0.65배), 최대 6체. 기본형 드래그 불가.
+메테오: 1.5초 낙하, 접촉 후 0.09초에 충돌 피해. 충돌 반경 1.75(Y 0.65배).
+장판 반경 1.25(Y 0.42배), 3.5초, 0.5초마다 피해 200%/총 7틱, 적 60% 감속. 메테오는 드래그 가능.</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>낙하와 충돌 전면</x:v>
+        <x:v>별빛·운석·폭발 전면 / 작은 파동·갈색 지면·붉은 균열 후면</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="76" customHeight="1">
@@ -4874,17 +4958,16 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="A9" s="27" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>적이 가장 많이 모인 지점 · 가장자리 안쪽 보정</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>착탄 지점 고정. 시전 마법진 없음.
-1.5초 가속 낙하, 접촉 후 0.09초에 피해. 잔열 2회.</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
+      <x:c r="B9" s="28" t="str">
+        <x:v>비활성 보존 ID</x:v>
+      </x:c>
+      <x:c r="C9" s="28" t="str">
+        <x:v>ID 3 기본 유성우 / 개화 메테오를 참조.</x:v>
+      </x:c>
+      <x:c r="D9" s="28" t="str">
         <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
       </x:c>
     </x:row>
@@ -4911,7 +4994,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe0ed84f3b1414b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4399e50245884bf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4972,7 +5055,7 @@
         <x:v>버전</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>게임 0.13.2 운영 개정 2026-09-20. 9종, ID 0–5·7–9. 삭제된 ID 6은 재사용하지 않습니다.</x:v>
+        <x:v>게임 0.14.0 운영 개정 2026-09-20. 활성 8종, ID 0–5·7·9. ID 6·8은 재사용하지 않습니다. 회색 ID 8 행은 통합 이력을 표시합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -4988,7 +5071,7 @@
         <x:v>공통 성장</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>직접 강화 E는 비전 지식으로 0~100, 각성 A는 동일 스킬 파편으로 0~10. A4/A8에 각각 1회 추가(화염 회오리는 2틱), A마다 효과량 +5%와 쿨타임 -2%. 운석은 고정 1회 충돌과 잔열 2회이며 타격 수 보너스를 사용하지 않습니다.</x:v>
+        <x:v>E 0~100은 비전 지식, A 0~10은 동일 스킬 파편. A4/A8 기본 타격 +1(화염 회오리 +2틱), A마다 효과량 +5%와 쿨타임 -2%. 메테오는 운석 1회와 3.5초 잔열로 고정됩니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
@@ -5012,7 +5095,7 @@
         <x:v>확률</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>전체 뽑기는 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 9종 스킬은 같은 확률(각 50%/9)입니다.</x:v>
+        <x:v>전체 스킬 50%, 비전 지식 10개 30%·20개 15%·50개 5%. 활성 8종은 각각 6.25%입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -5028,7 +5111,7 @@
         <x:v>투자 기간</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>각성 누적 55파편. 주당 21회 마탑 뽑기 기준으로 미보유 특정 스킬의 평균 개화 기간은 54회, 약 2.57주입니다. 기존 파편과 최초 보상은 제외합니다.</x:v>
+        <x:v>각성 누적 55파편. 미보유 특정 스킬은 해금 1회와 중복 2회가 필요하여 평균 48회, 주당 21회 기준 약 2.29주입니다. 기존 파편과 최초 보상은 제외합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
@@ -5036,7 +5119,7 @@
         <x:v>확률 편차</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>Acquisition의 P90은 정확한 음이항 계산입니다. 스킬당 95회까지 약 90%가 목표를 달성합니다. 천장이나 기간 보장은 없습니다.</x:v>
+        <x:v>미보유에서 개화까지의 P90은 음이항 계산 기준 84회입니다. 천장이나 기간 보장은 없습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5044,7 +5127,7 @@
         <x:v>특수 개화</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>천벌은 약 2초 예고 후 고정 반경 2.1 월드 단위 안 최대 10체를 공격합니다. 기기 비율이 피해 범위를 바꾸지 않습니다. Bloom의 최소·최대 반경은 모두 2.1입니다. 만년빙정은 시전 시작 시 유효 적 1체 여부로 단일/다수 형태를 선택합니다.</x:v>
+        <x:v>천벌: 2초 예고, 반경 2.1, 최대 10체. 만년빙정: 적 1체면 빙정, 다수면 8개×2회, 기절 없음. 메테오: 유성우 대신 거대 운석·3.5초 균열 장판·적 60% 감속. 세 형태 모두 A10에서 전환합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
@@ -5060,7 +5143,7 @@
         <x:v>개화 아이콘</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>개화 ON이면 BloomIcon을 사용합니다. 기본 실루엣과 구도를 유지하고 작은 발광·색조만 변화합니다. OFF 및 미해금 상태는 원본 아이콘을 사용합니다.</x:v>
+        <x:v>기본/개화 아이콘과 이름을 전환합니다. 일반 라이트닝은 세 가닥, 천벌은 기존 구도의 보라색 뇌운/낙뢰. 메테오는 운석과 뜨거운 균열, 만년빙정은 여러 송곳과 큰 중심 빙정입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" customHeight="1">
@@ -5068,7 +5151,7 @@
         <x:v>타격 연출</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>타격 시점에 피해·피격 반응·효과음을 맞춥니다. 별빛은 겹쳐 낙하하고 운석은 충돌 후 잔열을 남깁니다. 기절과 감속은 독립 만료하며 감속은 합산하지 않고 가장 강한 효과만 적용합니다. 전장 전환 시 진행 중인 타격과 이펙트를 취소합니다.</x:v>
+        <x:v>낙뢰마다 약한 흔들림, 천벌·메테오 충돌 시 절제된 강한 흔들림. 화면 흔들림 설정을 따르며 연속 흔들림을 합산하지 않습니다. 지속 장판·작은 착탄 파동은 후면입니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="84" customHeight="1">
@@ -5076,7 +5159,7 @@
         <x:v>외부 원본</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>ExternalAssets 원본은 보존합니다. 제작 출처: AI/comfyui/mage-vfx/revision1~5. 일반 라이트닝은 최초 ThunderEffects 원화 복원. 운석은 Comfy 표면 마스터를 회전·화염 흐름·파편 48프레임으로 가공했습니다.</x:v>
+        <x:v>ExternalAssets 원본 보존. 아트 공정 AI/comfyui/mage-vfx/revision1~6. v6은 기존 도트를 결정론적으로 재조합하고 Comfy의 색상 행렬·16색 양자화로 아이콘을 마감했습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -5100,7 +5183,7 @@
         <x:v>보류 개화</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>천벌·만년빙정 외 7종은 개화 미정이며 피해 또는 회복량이 15% 증가합니다.</x:v>
+        <x:v>천벌·만년빙정·메테오 외 5종은 전용 메커니즘 미정이며 피해 또는 회복량이 15% 증가합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="68" customHeight="1">
@@ -5124,7 +5207,7 @@
         <x:v>조준 구도</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>발 위치 기준 원형 게임 판정과 쿼터뷰 타원 장판 표시를 구분합니다. 분산 스킬인 얼음 송곳·유성우는 드래그 시전과 쿨다운 소비를 하지 않습니다.</x:v>
+        <x:v>유성우 기본형과 얼음 송곳은 드래그/쿨타임 소비가 없습니다. 메테오는 지점 시전 가능. 작은 파동·메테오 장판은 보이는 타원과 동일한 발 위치 판정을 사용합니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="68" customHeight="1">
@@ -5132,7 +5215,7 @@
         <x:v>각성 안내</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>A4/A8 추가 타격·틱, 다음 각성의 효과량·쿨타임·타격 수, A10 개화 효과를 상세 화면에 표시합니다. 운석은 추가 타격 보너스가 없습니다.</x:v>
+        <x:v>A4/A8 추가 타격·틱과 다음 각성 수치를 표시합니다. 메테오에는 유성우 기본형의 추가 낙하 수를 적용하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="68" customHeight="1">
@@ -5151,10 +5234,18 @@
         <x:v>핵심 VFX 목표 32px/월드 단위, 4~6색·Point·ASTC4×4. 단발 타격은 전면, 독 늪·잔열·흡인 등 지속 장판은 후면입니다. 이펙트가 큰 경우 원본 논리 해상도도 함께 높입니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="110" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>운석 통합</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>높은 E/A를 보존. 낮은 E의 실제 비전 지식 지출을 전액 환급, 낮은 A에 쓴 파편과 남은 파편을 합산. 둘 다 보유했으면 중복 보유 30파편 추가. 기존 내역을 보관하고 한 번만 적용. 기존 운석 슬롯은 유성우가 없을 때 교체하며, 이미 장착했다면 해당 슬롯만 비웁니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re36db18132344b88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaf48e4e26674f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Validate bloom overhaul on Android and correct skill detail values
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Skill_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Skill_Catalog.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R2b25563ab4234517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R252594dbfc684dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R9949f6ace02f4682"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="R55d581f3c3644ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R0397ae5074cf4a68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rdcad8e5da80041fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="Rf4e5a5af546e4974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Rbdb279aa60c54caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="1" r:id="R49790a27f37d4edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="2" r:id="R7bc3355c6b47471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloom" sheetId="3" r:id="R7859613883c44701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisition" sheetId="4" r:id="Rde563dac25514508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="5" r:id="R7e9539031e0b41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R1270c1c6fcee4214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targeting" sheetId="7" r:id="R1c48d1746ece4496"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Ra724209d916a4c30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="202" formatCode="0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -69,8 +69,13 @@
       <x:color rgb="FF6B7280"/>
       <x:name val="Malgun Gothic"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF6B7280"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +92,11 @@
         <x:fgColor rgb="FFE5E7EB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5E7EB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -94,7 +104,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -240,6 +250,31 @@
     <x:xf numFmtId="202" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -361,8 +396,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="Mage_Assets" displayName="Mage_Assets" ref="A1:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Mage_Assets" displayName="Mage_Assets" ref="A1:K10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="SkillId"/>
     <x:tableColumn id="2" name="Key"/>
     <x:tableColumn id="3" name="SkillAssetPath"/>
@@ -373,6 +408,7 @@
     <x:tableColumn id="8" name="SecondaryPrefabPath"/>
     <x:tableColumn id="9" name="BloomPrefabPath"/>
     <x:tableColumn id="10" name="BloomCastingPrefabPath"/>
+    <x:tableColumn id="11" name="BloomSecondaryPrefabPath"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -391,7 +427,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Mage_Guide" displayName="Mage_Guide" ref="A1:B22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="Mage_Guide" displayName="Mage_Guide" ref="A1:B29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Description"/>
@@ -842,31 +878,31 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="70" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="28" t="str">
+      <x:c r="C9" s="39" t="str">
         <x:v>독립 운석 삭제</x:v>
       </x:c>
-      <x:c r="D9" s="28" t="str">
+      <x:c r="D9" s="39" t="str">
         <x:v>ID 3 개화로 통합</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I9" s="28" t="str">
+      <x:c r="E9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="39" t="str">
         <x:v>ID 8은 비활성 보존 ID입니다. 로스터·장착·뽑기에 나오지 않으며 유성우의 개화 메테오로 통합했습니다.</x:v>
       </x:c>
     </x:row>
@@ -913,7 +949,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36a81b40f5f3428a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R361e8e086d3249e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1314,50 +1350,50 @@
       <x:c r="O8" s="5"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:f>'Skills'!B9</x:f>
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="32" t="n">
+      <x:c r="C9" s="40" t="n">
         <x:v>1.5499999523162842</x:v>
       </x:c>
-      <x:c r="D9" s="32" t="n">
+      <x:c r="D9" s="40" t="n">
         <x:v>0.800000011920929</x:v>
       </x:c>
-      <x:c r="E9" s="32" t="n">
+      <x:c r="E9" s="40" t="n">
         <x:v>0.800000011920929</x:v>
       </x:c>
-      <x:c r="F9" s="32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="32" t="n">
+      <x:c r="F9" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="40" t="n">
         <x:v>0.13461539149284363</x:v>
       </x:c>
-      <x:c r="I9" s="33" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="28" t="str">
+      <x:c r="I9" s="41" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="39" t="str">
         <x:v>충돌 1회 + 잔열 2회</x:v>
       </x:c>
-      <x:c r="K9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L9" s="27" t="n">
+      <x:c r="K9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="38" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="M9" s="27" t="n">
+      <x:c r="M9" s="38" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="N9" s="28" t="str">
+      <x:c r="N9" s="39" t="str">
         <x:v>Fire_Tornado_SFX</x:v>
       </x:c>
-      <x:c r="O9" s="28"/>
+      <x:c r="O9" s="39"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -1425,7 +1461,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05a404bc63e948f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9709b4067f404c24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1752,37 +1788,37 @@
       <x:c r="N8" s="5"/>
     </x:row>
     <x:row r="9" ht="90" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:f>'Skills'!C9</x:f>
         <x:v>독립 운석 삭제</x:v>
       </x:c>
-      <x:c r="C9" s="28" t="str">
+      <x:c r="C9" s="39" t="str">
         <x:v>통합됨</x:v>
       </x:c>
-      <x:c r="D9" s="28" t="str">
+      <x:c r="D9" s="39" t="str">
         <x:v>ID 3 메테오 개화 항목을 사용합니다.</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="n">
+      <x:c r="E9" s="38" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="n">
+      <x:c r="F9" s="38" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G9" s="27" t="n">
+      <x:c r="G9" s="38" t="n">
         <x:v>1.149999976158142</x:v>
       </x:c>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="28"/>
-      <x:c r="K9" s="28"/>
-      <x:c r="L9" s="28"/>
-      <x:c r="M9" s="28"/>
-      <x:c r="N9" s="28"/>
+      <x:c r="H9" s="39"/>
+      <x:c r="I9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="39"/>
+      <x:c r="K9" s="39"/>
+      <x:c r="L9" s="39"/>
+      <x:c r="M9" s="39"/>
+      <x:c r="N9" s="39"/>
     </x:row>
     <x:row r="10" ht="90" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -1836,7 +1872,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f09b68380e4338"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3cee35716e045c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2152,35 +2188,35 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:f>'Skills'!C9</x:f>
         <x:v>독립 운석 삭제</x:v>
       </x:c>
-      <x:c r="C9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="36" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="27" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="28" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I9" s="37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="27" t="n">
+      <x:c r="C9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="42" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2236,7 +2272,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e7c2d7649541c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23e47c6a2d6341fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4492,7 +4528,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e861d794534565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00f3df0dc3444bdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4753,32 +4789,32 @@
       <x:c r="K8" t="str"/>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:f>'Skills'!B9</x:f>
         <x:v>Meteor</x:v>
       </x:c>
-      <x:c r="C9" s="28" t="str">
+      <x:c r="C9" s="39" t="str">
         <x:v>Assets/MageTower/SO/Meteor/MageTowerSkill_Meteor.asset</x:v>
       </x:c>
-      <x:c r="D9" s="28" t="str">
+      <x:c r="D9" s="39" t="str">
         <x:v>Assets/_Project/Art/Icons/MageTower/Meteor.png</x:v>
       </x:c>
-      <x:c r="E9" s="28" t="str">
+      <x:c r="E9" s="39" t="str">
         <x:v>Assets/_Project/Art/Icons/MageTower/Meteor_Bloom.png</x:v>
       </x:c>
-      <x:c r="F9" s="28" t="str">
+      <x:c r="F9" s="39" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/Meteor.prefab</x:v>
       </x:c>
-      <x:c r="G9" s="28" t="str"/>
-      <x:c r="H9" s="28" t="str">
+      <x:c r="G9" s="39" t="str"/>
+      <x:c r="H9" s="39" t="str">
         <x:v>Assets/_Project/Prefabs/VFX/MageTower/MeteorCrater.prefab</x:v>
       </x:c>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="28"/>
-      <x:c r="K9" t="str"/>
+      <x:c r="I9" s="39"/>
+      <x:c r="J9" s="39"/>
+      <x:c r="K9" s="45" t="str"/>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="9" t="n">
@@ -4823,7 +4859,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ec304716b734fa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5faedbaba3e3420a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4958,16 +4994,16 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
-      <x:c r="A9" s="27" t="n">
+      <x:c r="A9" s="38" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="28" t="str">
+      <x:c r="B9" s="39" t="str">
         <x:v>비활성 보존 ID</x:v>
       </x:c>
-      <x:c r="C9" s="28" t="str">
+      <x:c r="C9" s="39" t="str">
         <x:v>ID 3 기본 유성우 / 개화 메테오를 참조.</x:v>
       </x:c>
-      <x:c r="D9" s="28" t="str">
+      <x:c r="D9" s="39" t="str">
         <x:v>운석과 폭발 전면 · 잔열 후면</x:v>
       </x:c>
     </x:row>
@@ -4994,7 +5030,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4399e50245884bf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f97ac94de5f41ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5245,7 +5281,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaf48e4e26674f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde8ed5ee0e8e465f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>